<commit_message>
Add Changdian Tech observation sample
</commit_message>
<xml_diff>
--- a/stock_review_template.xlsx
+++ b/stock_review_template.xlsx
@@ -190,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -257,6 +257,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -638,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -772,6 +790,34 @@
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t>每天不是“填满”就算完成，而是至少产出 1 条有效理由链。完整度检查有没有填，理由链质量检查有没有认真思考。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>长电科技10日样本数据说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>样本写入位置：每日观察!2:11，事后验证!2:8。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>个股数据：搜狐历史行情接口 cn_600584；大盘数据：搜狐历史行情接口 zs_000001；板块数据：东方财富半导体板块 BK1036。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>样本日期范围：2025-06-26 至 2025-07-09，共10个交易日；因当前接口未返回2026年数据，本样本按可取得的最近完整窗口填写。</t>
         </is>
       </c>
     </row>
@@ -982,511 +1028,1491 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="7">
         <f>IF(B2="","",TEXT(B2,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B2" s="8" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
-      <c r="H2" s="9" t="n"/>
-      <c r="I2" s="9" t="n"/>
-      <c r="J2" s="10" t="n"/>
-      <c r="K2" s="9" t="n"/>
-      <c r="L2" s="9" t="n"/>
-      <c r="M2" s="9" t="n"/>
-      <c r="N2" s="10" t="n"/>
-      <c r="O2" s="9" t="n"/>
-      <c r="P2" s="10" t="n"/>
-      <c r="Q2" s="10" t="n"/>
-      <c r="R2" s="9" t="n"/>
-      <c r="S2" s="10" t="n"/>
-      <c r="T2" s="10" t="n"/>
-      <c r="U2" s="11" t="n"/>
-      <c r="V2" s="11" t="n"/>
-      <c r="W2" s="12">
+      <c r="B2" s="25" t="n">
+        <v>45834</v>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>半导体/封测</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>震荡偏强</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>震荡</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>强于板块</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
+          <t>前高</t>
+        </is>
+      </c>
+      <c r="I2" s="10" t="inlineStr">
+        <is>
+          <t>33.30-33.40</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>6月25日前高33.30，今日最高33.40但收32.96，说明上方第一次出现分歧。</t>
+        </is>
+      </c>
+      <c r="K2" s="10" t="inlineStr">
+        <is>
+          <t>接近</t>
+        </is>
+      </c>
+      <c r="L2" s="10" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="M2" s="10" t="inlineStr">
+        <is>
+          <t>冲高回落</t>
+        </is>
+      </c>
+      <c r="N2" s="10" t="inlineStr">
+        <is>
+          <t>收32.96跌0.78%，盘中最高33.40触及前高区，成交量26.21万手；半导体跌1.17%，上证跌0.22%。</t>
+        </is>
+      </c>
+      <c r="O2" s="10" t="inlineStr">
+        <is>
+          <t>高位分歧</t>
+        </is>
+      </c>
+      <c r="P2" s="10" t="inlineStr">
+        <is>
+          <t>价格接近前高后没有收住，说明33.30-33.40附近存在短线抛压；但个股跌幅小于半导体，不能直接判定转弱。</t>
+        </is>
+      </c>
+      <c r="Q2" s="10" t="inlineStr">
+        <is>
+          <t>如果随后1-3日重新放量站上33.40，今天更像突破前正常分歧，而不是上攻失败。</t>
+        </is>
+      </c>
+      <c r="R2" s="10" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="S2" s="10" t="inlineStr">
+        <is>
+          <t>有明确前高和冲高回落事实，但板块当天较弱，单日不能确认失败。</t>
+        </is>
+      </c>
+      <c r="T2" s="10" t="inlineStr">
+        <is>
+          <t>后续只看是否收盘重新站上33.40。</t>
+        </is>
+      </c>
+      <c r="U2" s="11" t="inlineStr">
+        <is>
+          <t>前高区间确认、冲高回落与板块环境区分</t>
+        </is>
+      </c>
+      <c r="V2" s="11" t="inlineStr">
+        <is>
+          <t>数据源：搜狐历史行情个股；东方财富半导体板块；窗口为2025-06-26至2025-07-09。</t>
+        </is>
+      </c>
+      <c r="W2" s="26">
         <f>IF(B2="","",B2+3)</f>
         <v/>
       </c>
-      <c r="X2" s="12">
+      <c r="X2" s="26">
         <f>IF(B2="","",B2+5)</f>
         <v/>
       </c>
-      <c r="Y2" s="12">
+      <c r="Y2" s="26">
         <f>IF(B2="","",B2+10)</f>
         <v/>
       </c>
-      <c r="Z2" s="13">
+      <c r="Z2" s="27">
         <f>IF(B2="","",(--(B2&lt;&gt;"")+--(C2&lt;&gt;"")+--(D2&lt;&gt;"")+--(E2&lt;&gt;"")+--(F2&lt;&gt;"")+--(G2&lt;&gt;"")+--(H2&lt;&gt;"")+--(I2&lt;&gt;"")+--(J2&lt;&gt;"")+--(K2&lt;&gt;"")+--(L2&lt;&gt;"")+--(M2&lt;&gt;"")+--(N2&lt;&gt;"")+--(O2&lt;&gt;"")+--(P2&lt;&gt;"")+--(Q2&lt;&gt;"")+--(R2&lt;&gt;"")+--(S2&lt;&gt;"")+--(T2&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA2" s="16" t="n"/>
-      <c r="AB2" s="16" t="n"/>
-      <c r="AC2" s="16" t="n"/>
-      <c r="AD2" s="16" t="n"/>
+      <c r="AA2" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AB2" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AC2" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AD2" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
       <c r="AE2" s="7">
         <f>IF(B2="","",IF(AND(AA2="合格",AB2="合格",AC2="合格",AD2="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="72" customHeight="1">
       <c r="A3" s="7">
         <f>IF(B3="","",TEXT(B3,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B3" s="8" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="9" t="n"/>
-      <c r="E3" s="9" t="n"/>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="9" t="n"/>
-      <c r="H3" s="9" t="n"/>
-      <c r="I3" s="9" t="n"/>
-      <c r="J3" s="10" t="n"/>
-      <c r="K3" s="9" t="n"/>
-      <c r="L3" s="9" t="n"/>
-      <c r="M3" s="9" t="n"/>
-      <c r="N3" s="10" t="n"/>
-      <c r="O3" s="9" t="n"/>
-      <c r="P3" s="10" t="n"/>
-      <c r="Q3" s="10" t="n"/>
-      <c r="R3" s="9" t="n"/>
-      <c r="S3" s="10" t="n"/>
-      <c r="T3" s="10" t="n"/>
-      <c r="U3" s="11" t="n"/>
-      <c r="V3" s="11" t="n"/>
-      <c r="W3" s="12">
+      <c r="B3" s="25" t="n">
+        <v>45835</v>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>半导体/封测</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>震荡</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>轮动强势</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>强于板块</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>前高</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
+        <is>
+          <t>33.40</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>前一日最高33.40形成短线压力，今日最高34.08且收33.60。</t>
+        </is>
+      </c>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>突破</t>
+        </is>
+      </c>
+      <c r="L3" s="10" t="inlineStr">
+        <is>
+          <t>清晰</t>
+        </is>
+      </c>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>放量突破</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
+          <t>收33.60涨1.94%，最高34.08，成交量46.41万手明显放大；半导体涨1.08%，上证跌0.70%。</t>
+        </is>
+      </c>
+      <c r="O3" s="10" t="inlineStr">
+        <is>
+          <t>真突破/启动尝试</t>
+        </is>
+      </c>
+      <c r="P3" s="10" t="inlineStr">
+        <is>
+          <t>在大盘走弱时个股放量收过33.40，且强于半导体，说明有资金主动推动突破。</t>
+        </is>
+      </c>
+      <c r="Q3" s="10" t="inlineStr">
+        <is>
+          <t>收盘离日高较远，若很快跌回33.40下方并放量，突破解释会削弱。</t>
+        </is>
+      </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>量价与相对强弱都支持，但只是一日突破，还没有回踩确认。</t>
+        </is>
+      </c>
+      <c r="T3" s="10" t="inlineStr">
+        <is>
+          <t>后续只看是否守住33.30-33.40。</t>
+        </is>
+      </c>
+      <c r="U3" s="11" t="inlineStr">
+        <is>
+          <t>突破有效性、放量含义、回踩确认</t>
+        </is>
+      </c>
+      <c r="V3" s="11" t="inlineStr">
+        <is>
+          <t>这是突破尝试，不等于已经进入主升。</t>
+        </is>
+      </c>
+      <c r="W3" s="26">
         <f>IF(B3="","",B3+3)</f>
         <v/>
       </c>
-      <c r="X3" s="12">
+      <c r="X3" s="26">
         <f>IF(B3="","",B3+5)</f>
         <v/>
       </c>
-      <c r="Y3" s="12">
+      <c r="Y3" s="26">
         <f>IF(B3="","",B3+10)</f>
         <v/>
       </c>
-      <c r="Z3" s="13">
+      <c r="Z3" s="27">
         <f>IF(B3="","",(--(B3&lt;&gt;"")+--(C3&lt;&gt;"")+--(D3&lt;&gt;"")+--(E3&lt;&gt;"")+--(F3&lt;&gt;"")+--(G3&lt;&gt;"")+--(H3&lt;&gt;"")+--(I3&lt;&gt;"")+--(J3&lt;&gt;"")+--(K3&lt;&gt;"")+--(L3&lt;&gt;"")+--(M3&lt;&gt;"")+--(N3&lt;&gt;"")+--(O3&lt;&gt;"")+--(P3&lt;&gt;"")+--(Q3&lt;&gt;"")+--(R3&lt;&gt;"")+--(S3&lt;&gt;"")+--(T3&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA3" s="16" t="n"/>
-      <c r="AB3" s="16" t="n"/>
-      <c r="AC3" s="16" t="n"/>
-      <c r="AD3" s="16" t="n"/>
+      <c r="AA3" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AB3" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AC3" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AD3" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
       <c r="AE3" s="7">
         <f>IF(B3="","",IF(AND(AA3="合格",AB3="合格",AC3="合格",AD3="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="72" customHeight="1">
       <c r="A4" s="7">
         <f>IF(B4="","",TEXT(B4,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="9" t="n"/>
-      <c r="E4" s="9" t="n"/>
-      <c r="F4" s="9" t="n"/>
-      <c r="G4" s="9" t="n"/>
-      <c r="H4" s="9" t="n"/>
-      <c r="I4" s="9" t="n"/>
-      <c r="J4" s="10" t="n"/>
-      <c r="K4" s="9" t="n"/>
-      <c r="L4" s="9" t="n"/>
-      <c r="M4" s="9" t="n"/>
-      <c r="N4" s="10" t="n"/>
-      <c r="O4" s="9" t="n"/>
-      <c r="P4" s="10" t="n"/>
-      <c r="Q4" s="10" t="n"/>
-      <c r="R4" s="9" t="n"/>
-      <c r="S4" s="10" t="n"/>
-      <c r="T4" s="10" t="n"/>
-      <c r="U4" s="11" t="n"/>
-      <c r="V4" s="11" t="n"/>
-      <c r="W4" s="12">
+      <c r="B4" s="25" t="n">
+        <v>45838</v>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>半导体/封测</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>震荡偏强</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>主线强势</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>弱于板块</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>前高</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>34.08</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>6月27日突破日最高34.08是新的短线观察压力。</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>接近</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>横盘震荡</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="inlineStr">
+        <is>
+          <t>收33.69涨0.27%，成交量30.02万手缩小；半导体涨1.67%，上证涨0.59%。</t>
+        </is>
+      </c>
+      <c r="O4" s="10" t="inlineStr">
+        <is>
+          <t>震荡整理</t>
+        </is>
+      </c>
+      <c r="P4" s="10" t="inlineStr">
+        <is>
+          <t>突破后没有继续放量上攻，只是在33.40上方小幅整理；但弱于强势板块，说明主动性不足。</t>
+        </is>
+      </c>
+      <c r="Q4" s="10" t="inlineStr">
+        <is>
+          <t>如果次日放量站上34.08，则今天的缩量可能只是突破后的蓄势。</t>
+        </is>
+      </c>
+      <c r="R4" s="10" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="S4" s="10" t="inlineStr">
+        <is>
+          <t>事实更多指向整理，但是否转弱还缺少跌破关键位。</t>
+        </is>
+      </c>
+      <c r="T4" s="10" t="inlineStr">
+        <is>
+          <t>后续只看是否收盘站上34.08。</t>
+        </is>
+      </c>
+      <c r="U4" s="11" t="inlineStr">
+        <is>
+          <t>突破后缩量整理、相对板块弱势识别</t>
+        </is>
+      </c>
+      <c r="V4" s="11" t="inlineStr">
+        <is>
+          <t>这一天的重点不是预测涨跌，而是识别“突破后没有立刻延续”。</t>
+        </is>
+      </c>
+      <c r="W4" s="26">
         <f>IF(B4="","",B4+3)</f>
         <v/>
       </c>
-      <c r="X4" s="12">
+      <c r="X4" s="26">
         <f>IF(B4="","",B4+5)</f>
         <v/>
       </c>
-      <c r="Y4" s="12">
+      <c r="Y4" s="26">
         <f>IF(B4="","",B4+10)</f>
         <v/>
       </c>
-      <c r="Z4" s="13">
+      <c r="Z4" s="27">
         <f>IF(B4="","",(--(B4&lt;&gt;"")+--(C4&lt;&gt;"")+--(D4&lt;&gt;"")+--(E4&lt;&gt;"")+--(F4&lt;&gt;"")+--(G4&lt;&gt;"")+--(H4&lt;&gt;"")+--(I4&lt;&gt;"")+--(J4&lt;&gt;"")+--(K4&lt;&gt;"")+--(L4&lt;&gt;"")+--(M4&lt;&gt;"")+--(N4&lt;&gt;"")+--(O4&lt;&gt;"")+--(P4&lt;&gt;"")+--(Q4&lt;&gt;"")+--(R4&lt;&gt;"")+--(S4&lt;&gt;"")+--(T4&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA4" s="16" t="n"/>
-      <c r="AB4" s="16" t="n"/>
-      <c r="AC4" s="16" t="n"/>
-      <c r="AD4" s="16" t="n"/>
+      <c r="AA4" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AB4" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AC4" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AD4" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
       <c r="AE4" s="7">
         <f>IF(B4="","",IF(AND(AA4="合格",AB4="合格",AC4="合格",AD4="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="7">
         <f>IF(B5="","",TEXT(B5,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="9" t="n"/>
-      <c r="I5" s="9" t="n"/>
-      <c r="J5" s="10" t="n"/>
-      <c r="K5" s="9" t="n"/>
-      <c r="L5" s="9" t="n"/>
-      <c r="M5" s="9" t="n"/>
-      <c r="N5" s="10" t="n"/>
-      <c r="O5" s="9" t="n"/>
-      <c r="P5" s="10" t="n"/>
-      <c r="Q5" s="10" t="n"/>
-      <c r="R5" s="9" t="n"/>
-      <c r="S5" s="10" t="n"/>
-      <c r="T5" s="10" t="n"/>
-      <c r="U5" s="11" t="n"/>
-      <c r="V5" s="11" t="n"/>
-      <c r="W5" s="12">
+      <c r="B5" s="25" t="n">
+        <v>45839</v>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>半导体/封测</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>震荡偏强</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>轮动强势</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>强于板块</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>前高</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>34.08</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>6月27日高点34.08被盘中突破，但收盘33.97没有站上。</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>站上未确认</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>清晰</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>高位放量震荡</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr">
+        <is>
+          <t>收33.97涨0.83%，盘中最高34.38创短线新高，成交量39.29万手；半导体涨0.33%，上证涨0.39%。</t>
+        </is>
+      </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>高位分歧</t>
+        </is>
+      </c>
+      <c r="P5" s="10" t="inlineStr">
+        <is>
+          <t>盘中新高但收回34.08下方，说明新高位置有抛压；不过个股仍强于板块，不能直接判定见顶。</t>
+        </is>
+      </c>
+      <c r="Q5" s="10" t="inlineStr">
+        <is>
+          <t>如果后续收盘站回34.08并继续放量，新高回落可能只是分歧换手。</t>
+        </is>
+      </c>
+      <c r="R5" s="10" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="S5" s="10" t="inlineStr">
+        <is>
+          <t>关键位清晰且有冲高回落，但趋势尚未破坏。</t>
+        </is>
+      </c>
+      <c r="T5" s="10" t="inlineStr">
+        <is>
+          <t>后续只看是否收盘站上34.08。</t>
+        </is>
+      </c>
+      <c r="U5" s="11" t="inlineStr">
+        <is>
+          <t>盘中新高与收盘确认、分歧换手</t>
+        </is>
+      </c>
+      <c r="V5" s="11" t="inlineStr">
+        <is>
+          <t>这是判断“真突破还是假突破”的典型样本。</t>
+        </is>
+      </c>
+      <c r="W5" s="26">
         <f>IF(B5="","",B5+3)</f>
         <v/>
       </c>
-      <c r="X5" s="12">
+      <c r="X5" s="26">
         <f>IF(B5="","",B5+5)</f>
         <v/>
       </c>
-      <c r="Y5" s="12">
+      <c r="Y5" s="26">
         <f>IF(B5="","",B5+10)</f>
         <v/>
       </c>
-      <c r="Z5" s="13">
+      <c r="Z5" s="27">
         <f>IF(B5="","",(--(B5&lt;&gt;"")+--(C5&lt;&gt;"")+--(D5&lt;&gt;"")+--(E5&lt;&gt;"")+--(F5&lt;&gt;"")+--(G5&lt;&gt;"")+--(H5&lt;&gt;"")+--(I5&lt;&gt;"")+--(J5&lt;&gt;"")+--(K5&lt;&gt;"")+--(L5&lt;&gt;"")+--(M5&lt;&gt;"")+--(N5&lt;&gt;"")+--(O5&lt;&gt;"")+--(P5&lt;&gt;"")+--(Q5&lt;&gt;"")+--(R5&lt;&gt;"")+--(S5&lt;&gt;"")+--(T5&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA5" s="16" t="n"/>
-      <c r="AB5" s="16" t="n"/>
-      <c r="AC5" s="16" t="n"/>
-      <c r="AD5" s="16" t="n"/>
+      <c r="AA5" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AB5" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AC5" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AD5" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
       <c r="AE5" s="7">
         <f>IF(B5="","",IF(AND(AA5="合格",AB5="合格",AC5="合格",AD5="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="72" customHeight="1">
       <c r="A6" s="7">
         <f>IF(B6="","",TEXT(B6,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="n"/>
-      <c r="J6" s="10" t="n"/>
-      <c r="K6" s="9" t="n"/>
-      <c r="L6" s="9" t="n"/>
-      <c r="M6" s="9" t="n"/>
-      <c r="N6" s="10" t="n"/>
-      <c r="O6" s="9" t="n"/>
-      <c r="P6" s="10" t="n"/>
-      <c r="Q6" s="10" t="n"/>
-      <c r="R6" s="9" t="n"/>
-      <c r="S6" s="10" t="n"/>
-      <c r="T6" s="10" t="n"/>
-      <c r="U6" s="11" t="n"/>
-      <c r="V6" s="11" t="n"/>
-      <c r="W6" s="12">
+      <c r="B6" s="25" t="n">
+        <v>45840</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>半导体/封测</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>震荡</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>退潮</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>强于板块</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>大阳线低点</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>33.00-33.30</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>6月27日放量阳线低点33.00，6月25日前高33.30附近构成回踩观察区。</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>回踩</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>缩量回调</t>
+        </is>
+      </c>
+      <c r="N6" s="10" t="inlineStr">
+        <is>
+          <t>收33.31跌1.94%，最低33.23，成交量26.21万手；半导体跌2.18%，上证跌0.09%。</t>
+        </is>
+      </c>
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t>健康回调</t>
+        </is>
+      </c>
+      <c r="P6" s="10" t="inlineStr">
+        <is>
+          <t>价格回到33.00-33.30支撑区附近但没有明显放量跌破，且跌幅小于半导体，暂时更像突破后的回踩。</t>
+        </is>
+      </c>
+      <c r="Q6" s="10" t="inlineStr">
+        <is>
+          <t>如果随后跌破33.00并收不回，健康回调解释会被证伪。</t>
+        </is>
+      </c>
+      <c r="R6" s="10" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="S6" s="10" t="inlineStr">
+        <is>
+          <t>回踩区间是人工划出来的，不够精确，只能作为低强度假设。</t>
+        </is>
+      </c>
+      <c r="T6" s="10" t="inlineStr">
+        <is>
+          <t>后续只看是否跌破33.00。</t>
+        </is>
+      </c>
+      <c r="U6" s="11" t="inlineStr">
+        <is>
+          <t>大阳线低点、支撑区间而非单点、缩量回调</t>
+        </is>
+      </c>
+      <c r="V6" s="11" t="inlineStr">
+        <is>
+          <t>这行故意保持低判断强度，因为支撑区不是非常清晰。</t>
+        </is>
+      </c>
+      <c r="W6" s="26">
         <f>IF(B6="","",B6+3)</f>
         <v/>
       </c>
-      <c r="X6" s="12">
+      <c r="X6" s="26">
         <f>IF(B6="","",B6+5)</f>
         <v/>
       </c>
-      <c r="Y6" s="12">
+      <c r="Y6" s="26">
         <f>IF(B6="","",B6+10)</f>
         <v/>
       </c>
-      <c r="Z6" s="13">
+      <c r="Z6" s="27">
         <f>IF(B6="","",(--(B6&lt;&gt;"")+--(C6&lt;&gt;"")+--(D6&lt;&gt;"")+--(E6&lt;&gt;"")+--(F6&lt;&gt;"")+--(G6&lt;&gt;"")+--(H6&lt;&gt;"")+--(I6&lt;&gt;"")+--(J6&lt;&gt;"")+--(K6&lt;&gt;"")+--(L6&lt;&gt;"")+--(M6&lt;&gt;"")+--(N6&lt;&gt;"")+--(O6&lt;&gt;"")+--(P6&lt;&gt;"")+--(Q6&lt;&gt;"")+--(R6&lt;&gt;"")+--(S6&lt;&gt;"")+--(T6&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA6" s="16" t="n"/>
-      <c r="AB6" s="16" t="n"/>
-      <c r="AC6" s="16" t="n"/>
-      <c r="AD6" s="16" t="n"/>
+      <c r="AA6" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AB6" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AC6" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AD6" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
       <c r="AE6" s="7">
         <f>IF(B6="","",IF(AND(AA6="合格",AB6="合格",AC6="合格",AD6="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="72" customHeight="1">
       <c r="A7" s="7">
         <f>IF(B7="","",TEXT(B7,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
-      <c r="I7" s="9" t="n"/>
-      <c r="J7" s="10" t="n"/>
-      <c r="K7" s="9" t="n"/>
-      <c r="L7" s="9" t="n"/>
-      <c r="M7" s="9" t="n"/>
-      <c r="N7" s="10" t="n"/>
-      <c r="O7" s="9" t="n"/>
-      <c r="P7" s="10" t="n"/>
-      <c r="Q7" s="10" t="n"/>
-      <c r="R7" s="9" t="n"/>
-      <c r="S7" s="10" t="n"/>
-      <c r="T7" s="10" t="n"/>
-      <c r="U7" s="11" t="n"/>
-      <c r="V7" s="11" t="n"/>
-      <c r="W7" s="12">
+      <c r="B7" s="25" t="n">
+        <v>45841</v>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>半导体/封测</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>震荡偏强</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>震荡</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>强于板块</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>箱体下沿</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>33.20-33.30</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>7月2日低点33.23与7月3日低点33.23重合，形成短线震荡下沿。</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>回踩</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>回踩支撑不破</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
+        <is>
+          <t>收33.53涨0.66%，最低33.23再次守住，成交量21.32万手继续缩小；半导体涨0.36%，上证涨0.18%。</t>
+        </is>
+      </c>
+      <c r="O7" s="10" t="inlineStr">
+        <is>
+          <t>震荡整理</t>
+        </is>
+      </c>
+      <c r="P7" s="10" t="inlineStr">
+        <is>
+          <t>同一低点附近两次守住，价格没有继续向下；但成交量缩小，说明反弹力度也不强。</t>
+        </is>
+      </c>
+      <c r="Q7" s="10" t="inlineStr">
+        <is>
+          <t>如果后续跌破33.20，所谓箱体下沿就只是临时巧合。</t>
+        </is>
+      </c>
+      <c r="R7" s="10" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="S7" s="10" t="inlineStr">
+        <is>
+          <t>只有两个交易日的低点，结构证据偏少。</t>
+        </is>
+      </c>
+      <c r="T7" s="10" t="inlineStr">
+        <is>
+          <t>后续只看是否跌破33.20。</t>
+        </is>
+      </c>
+      <c r="U7" s="11" t="inlineStr">
+        <is>
+          <t>箱体下沿需要多次确认、缩量反弹强弱</t>
+        </is>
+      </c>
+      <c r="V7" s="11" t="inlineStr">
+        <is>
+          <t>这是一条“暂时结构”，不是强结论。</t>
+        </is>
+      </c>
+      <c r="W7" s="26">
         <f>IF(B7="","",B7+3)</f>
         <v/>
       </c>
-      <c r="X7" s="12">
+      <c r="X7" s="26">
         <f>IF(B7="","",B7+5)</f>
         <v/>
       </c>
-      <c r="Y7" s="12">
+      <c r="Y7" s="26">
         <f>IF(B7="","",B7+10)</f>
         <v/>
       </c>
-      <c r="Z7" s="13">
+      <c r="Z7" s="27">
         <f>IF(B7="","",(--(B7&lt;&gt;"")+--(C7&lt;&gt;"")+--(D7&lt;&gt;"")+--(E7&lt;&gt;"")+--(F7&lt;&gt;"")+--(G7&lt;&gt;"")+--(H7&lt;&gt;"")+--(I7&lt;&gt;"")+--(J7&lt;&gt;"")+--(K7&lt;&gt;"")+--(L7&lt;&gt;"")+--(M7&lt;&gt;"")+--(N7&lt;&gt;"")+--(O7&lt;&gt;"")+--(P7&lt;&gt;"")+--(Q7&lt;&gt;"")+--(R7&lt;&gt;"")+--(S7&lt;&gt;"")+--(T7&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA7" s="16" t="n"/>
-      <c r="AB7" s="16" t="n"/>
-      <c r="AC7" s="16" t="n"/>
-      <c r="AD7" s="16" t="n"/>
+      <c r="AA7" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AB7" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AC7" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AD7" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
       <c r="AE7" s="7">
         <f>IF(B7="","",IF(AND(AA7="合格",AB7="合格",AC7="合格",AD7="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="72" customHeight="1">
       <c r="A8" s="7">
         <f>IF(B8="","",TEXT(B8,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="10" t="n"/>
-      <c r="K8" s="9" t="n"/>
-      <c r="L8" s="9" t="n"/>
-      <c r="M8" s="9" t="n"/>
-      <c r="N8" s="10" t="n"/>
-      <c r="O8" s="9" t="n"/>
-      <c r="P8" s="10" t="n"/>
-      <c r="Q8" s="10" t="n"/>
-      <c r="R8" s="9" t="n"/>
-      <c r="S8" s="10" t="n"/>
-      <c r="T8" s="10" t="n"/>
-      <c r="U8" s="11" t="n"/>
-      <c r="V8" s="11" t="n"/>
-      <c r="W8" s="12">
+      <c r="B8" s="25" t="n">
+        <v>45842</v>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>半导体/封测</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>震荡偏强</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>震荡</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>同步板块</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>箱体下沿</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>33.20-33.30</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>前两日33.23低点形成短线下沿，今日收33.23正好回到下沿。</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>接近</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>横盘震荡</t>
+        </is>
+      </c>
+      <c r="N8" s="10" t="inlineStr">
+        <is>
+          <t>收33.23跌0.89%，最低33.10，成交量20.30万手；半导体跌0.93%，上证涨0.32%。</t>
+        </is>
+      </c>
+      <c r="O8" s="10" t="inlineStr">
+        <is>
+          <t>震荡整理</t>
+        </is>
+      </c>
+      <c r="P8" s="10" t="inlineStr">
+        <is>
+          <t>价格回到下沿附近但没有放量大跌，仍可能是箱体震荡；不过大盘上涨时个股不涨，主动性偏弱。</t>
+        </is>
+      </c>
+      <c r="Q8" s="10" t="inlineStr">
+        <is>
+          <t>如果下一日跌破33.00，震荡整理会转向突破失败或转弱。</t>
+        </is>
+      </c>
+      <c r="R8" s="10" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="S8" s="10" t="inlineStr">
+        <is>
+          <t>位置接近支撑但没有明确反包或放量，结论只能低强度。</t>
+        </is>
+      </c>
+      <c r="T8" s="10" t="inlineStr">
+        <is>
+          <t>后续只看是否跌破33.00。</t>
+        </is>
+      </c>
+      <c r="U8" s="11" t="inlineStr">
+        <is>
+          <t>弱于大盘的含义、箱体下沿有效性</t>
+        </is>
+      </c>
+      <c r="V8" s="11" t="inlineStr">
+        <is>
+          <t>这里更适合观察，不适合急着下强判断。</t>
+        </is>
+      </c>
+      <c r="W8" s="26">
         <f>IF(B8="","",B8+3)</f>
         <v/>
       </c>
-      <c r="X8" s="12">
+      <c r="X8" s="26">
         <f>IF(B8="","",B8+5)</f>
         <v/>
       </c>
-      <c r="Y8" s="12">
+      <c r="Y8" s="26">
         <f>IF(B8="","",B8+10)</f>
         <v/>
       </c>
-      <c r="Z8" s="13">
+      <c r="Z8" s="27">
         <f>IF(B8="","",(--(B8&lt;&gt;"")+--(C8&lt;&gt;"")+--(D8&lt;&gt;"")+--(E8&lt;&gt;"")+--(F8&lt;&gt;"")+--(G8&lt;&gt;"")+--(H8&lt;&gt;"")+--(I8&lt;&gt;"")+--(J8&lt;&gt;"")+--(K8&lt;&gt;"")+--(L8&lt;&gt;"")+--(M8&lt;&gt;"")+--(N8&lt;&gt;"")+--(O8&lt;&gt;"")+--(P8&lt;&gt;"")+--(Q8&lt;&gt;"")+--(R8&lt;&gt;"")+--(S8&lt;&gt;"")+--(T8&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA8" s="16" t="n"/>
-      <c r="AB8" s="16" t="n"/>
-      <c r="AC8" s="16" t="n"/>
-      <c r="AD8" s="16" t="n"/>
+      <c r="AA8" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AB8" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AC8" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AD8" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
       <c r="AE8" s="7">
         <f>IF(B8="","",IF(AND(AA8="合格",AB8="合格",AC8="合格",AD8="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="7">
         <f>IF(B9="","",TEXT(B9,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n"/>
-      <c r="J9" s="10" t="n"/>
-      <c r="K9" s="9" t="n"/>
-      <c r="L9" s="9" t="n"/>
-      <c r="M9" s="9" t="n"/>
-      <c r="N9" s="10" t="n"/>
-      <c r="O9" s="9" t="n"/>
-      <c r="P9" s="10" t="n"/>
-      <c r="Q9" s="10" t="n"/>
-      <c r="R9" s="9" t="n"/>
-      <c r="S9" s="10" t="n"/>
-      <c r="T9" s="10" t="n"/>
-      <c r="U9" s="11" t="n"/>
-      <c r="V9" s="11" t="n"/>
-      <c r="W9" s="12">
+      <c r="B9" s="25" t="n">
+        <v>45845</v>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>半导体/封测</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>震荡偏强</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>震荡</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>弱于板块</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>大阳线低点</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>33.00</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>6月27日放量阳线低点33.00，此前也作为回踩观察位。</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>跌破</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>清晰</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>跌破关键位</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>收32.95跌0.84%，最低32.88，跌破33.00，成交量15.46万手；半导体跌0.13%，上证微涨0.02%。</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>退潮转弱</t>
+        </is>
+      </c>
+      <c r="P9" s="10" t="inlineStr">
+        <is>
+          <t>在板块和大盘没有明显下跌时，个股跌破33.00关键位，说明前期突破结构被破坏。</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>如果下一两日快速收回33.30上方，今天可能是假跌破。</t>
+        </is>
+      </c>
+      <c r="R9" s="10" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="S9" s="10" t="inlineStr">
+        <is>
+          <t>关键位清晰，且相对板块转弱，但缩量下跌意味着杀跌并不充分。</t>
+        </is>
+      </c>
+      <c r="T9" s="10" t="inlineStr">
+        <is>
+          <t>后续只看是否收回33.30。</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>跌破关键位、假跌破识别、相对弱势</t>
+        </is>
+      </c>
+      <c r="V9" s="11" t="inlineStr">
+        <is>
+          <t>这一天是从“支撑观察”转为“结构受损观察”的分界。</t>
+        </is>
+      </c>
+      <c r="W9" s="26">
         <f>IF(B9="","",B9+3)</f>
         <v/>
       </c>
-      <c r="X9" s="12">
+      <c r="X9" s="26">
         <f>IF(B9="","",B9+5)</f>
         <v/>
       </c>
-      <c r="Y9" s="12">
+      <c r="Y9" s="26">
         <f>IF(B9="","",B9+10)</f>
         <v/>
       </c>
-      <c r="Z9" s="13">
+      <c r="Z9" s="27">
         <f>IF(B9="","",(--(B9&lt;&gt;"")+--(C9&lt;&gt;"")+--(D9&lt;&gt;"")+--(E9&lt;&gt;"")+--(F9&lt;&gt;"")+--(G9&lt;&gt;"")+--(H9&lt;&gt;"")+--(I9&lt;&gt;"")+--(J9&lt;&gt;"")+--(K9&lt;&gt;"")+--(L9&lt;&gt;"")+--(M9&lt;&gt;"")+--(N9&lt;&gt;"")+--(O9&lt;&gt;"")+--(P9&lt;&gt;"")+--(Q9&lt;&gt;"")+--(R9&lt;&gt;"")+--(S9&lt;&gt;"")+--(T9&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA9" s="16" t="n"/>
-      <c r="AB9" s="16" t="n"/>
-      <c r="AC9" s="16" t="n"/>
-      <c r="AD9" s="16" t="n"/>
+      <c r="AA9" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AB9" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AC9" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AD9" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
       <c r="AE9" s="7">
         <f>IF(B9="","",IF(AND(AA9="合格",AB9="合格",AC9="合格",AD9="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="72" customHeight="1">
       <c r="A10" s="7">
         <f>IF(B10="","",TEXT(B10,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="n"/>
-      <c r="J10" s="10" t="n"/>
-      <c r="K10" s="9" t="n"/>
-      <c r="L10" s="9" t="n"/>
-      <c r="M10" s="9" t="n"/>
-      <c r="N10" s="10" t="n"/>
-      <c r="O10" s="9" t="n"/>
-      <c r="P10" s="10" t="n"/>
-      <c r="Q10" s="10" t="n"/>
-      <c r="R10" s="9" t="n"/>
-      <c r="S10" s="10" t="n"/>
-      <c r="T10" s="10" t="n"/>
-      <c r="U10" s="11" t="n"/>
-      <c r="V10" s="11" t="n"/>
-      <c r="W10" s="12">
+      <c r="B10" s="25" t="n">
+        <v>45846</v>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>半导体/封测</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>上升</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>轮动强势</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>同步板块</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>前高</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>33.30-33.40</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>跌破33.00后快速收回，33.30-33.40重新变成修复确认位。</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>跌破后收回</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>低位反弹</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>收33.55涨1.82%，最低33.01后收回33.30-33.40，成交量24.45万手；半导体涨1.50%，上证涨0.70%。</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>弱反弹</t>
+        </is>
+      </c>
+      <c r="P10" s="10" t="inlineStr">
+        <is>
+          <t>价格收回关键位说明7月7日跌破没有继续恶化，但反弹主要伴随大盘和板块转强，暂不能认定重新启动。</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>如果后续不能继续站稳33.40并上攻33.80，反弹仍可能只是箱体震荡的一部分。</t>
+        </is>
+      </c>
+      <c r="R10" s="10" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="S10" s="10" t="inlineStr">
+        <is>
+          <t>修复动作明确，但外部环境同步转强，个股独立性不足。</t>
+        </is>
+      </c>
+      <c r="T10" s="10" t="inlineStr">
+        <is>
+          <t>后续只看是否连续收在33.40上方。</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>跌破后收回、修复与重新启动区别</t>
+        </is>
+      </c>
+      <c r="V10" s="11" t="inlineStr">
+        <is>
+          <t>不要因为一天大涨就把它重新判成强趋势。</t>
+        </is>
+      </c>
+      <c r="W10" s="26">
         <f>IF(B10="","",B10+3)</f>
         <v/>
       </c>
-      <c r="X10" s="12">
+      <c r="X10" s="26">
         <f>IF(B10="","",B10+5)</f>
         <v/>
       </c>
-      <c r="Y10" s="12">
+      <c r="Y10" s="26">
         <f>IF(B10="","",B10+10)</f>
         <v/>
       </c>
-      <c r="Z10" s="13">
+      <c r="Z10" s="27">
         <f>IF(B10="","",(--(B10&lt;&gt;"")+--(C10&lt;&gt;"")+--(D10&lt;&gt;"")+--(E10&lt;&gt;"")+--(F10&lt;&gt;"")+--(G10&lt;&gt;"")+--(H10&lt;&gt;"")+--(I10&lt;&gt;"")+--(J10&lt;&gt;"")+--(K10&lt;&gt;"")+--(L10&lt;&gt;"")+--(M10&lt;&gt;"")+--(N10&lt;&gt;"")+--(O10&lt;&gt;"")+--(P10&lt;&gt;"")+--(Q10&lt;&gt;"")+--(R10&lt;&gt;"")+--(S10&lt;&gt;"")+--(T10&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA10" s="16" t="n"/>
-      <c r="AB10" s="16" t="n"/>
-      <c r="AC10" s="16" t="n"/>
-      <c r="AD10" s="16" t="n"/>
+      <c r="AA10" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AB10" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AC10" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AD10" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
       <c r="AE10" s="7">
         <f>IF(B10="","",IF(AND(AA10="合格",AB10="合格",AC10="合格",AD10="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="72" customHeight="1">
       <c r="A11" s="7">
         <f>IF(B11="","",TEXT(B11,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="9" t="n"/>
-      <c r="H11" s="9" t="n"/>
-      <c r="I11" s="9" t="n"/>
-      <c r="J11" s="10" t="n"/>
-      <c r="K11" s="9" t="n"/>
-      <c r="L11" s="9" t="n"/>
-      <c r="M11" s="9" t="n"/>
-      <c r="N11" s="10" t="n"/>
-      <c r="O11" s="9" t="n"/>
-      <c r="P11" s="10" t="n"/>
-      <c r="Q11" s="10" t="n"/>
-      <c r="R11" s="9" t="n"/>
-      <c r="S11" s="10" t="n"/>
-      <c r="T11" s="10" t="n"/>
-      <c r="U11" s="11" t="n"/>
-      <c r="V11" s="11" t="n"/>
-      <c r="W11" s="12">
+      <c r="B11" s="25" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>半导体/封测</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>震荡偏强</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>震荡</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>同步板块</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>箱体下沿</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>33.00-33.20</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>近几日低点集中在33.00-33.20，当前仍围绕这个区域反复。</t>
+        </is>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>接近</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>横盘震荡</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>收33.18跌1.10%，最低33.10，成交量19.43万手；半导体跌1.12%，上证跌0.13%。</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>震荡整理</t>
+        </is>
+      </c>
+      <c r="P11" s="10" t="inlineStr">
+        <is>
+          <t>价格没有继续向上确认33.40，也没有有效跌破33.00，说明短线仍在33.00-34.08之间震荡。</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>如果后续放量跌破33.00，震荡整理会转为转弱；若放量站上34.08，才说明重新转强。</t>
+        </is>
+      </c>
+      <c r="R11" s="10" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="S11" s="10" t="inlineStr">
+        <is>
+          <t>上下边界都有，但当前价格在中低位，方向信息不足。</t>
+        </is>
+      </c>
+      <c r="T11" s="10" t="inlineStr">
+        <is>
+          <t>后续只看33.00是否被有效跌破。</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>箱体边界、方向未明时降低判断强度</t>
+        </is>
+      </c>
+      <c r="V11" s="11" t="inlineStr">
+        <is>
+          <t>这是一个“看不清就承认看不清”的样本。</t>
+        </is>
+      </c>
+      <c r="W11" s="26">
         <f>IF(B11="","",B11+3)</f>
         <v/>
       </c>
-      <c r="X11" s="12">
+      <c r="X11" s="26">
         <f>IF(B11="","",B11+5)</f>
         <v/>
       </c>
-      <c r="Y11" s="12">
+      <c r="Y11" s="26">
         <f>IF(B11="","",B11+10)</f>
         <v/>
       </c>
-      <c r="Z11" s="13">
+      <c r="Z11" s="27">
         <f>IF(B11="","",(--(B11&lt;&gt;"")+--(C11&lt;&gt;"")+--(D11&lt;&gt;"")+--(E11&lt;&gt;"")+--(F11&lt;&gt;"")+--(G11&lt;&gt;"")+--(H11&lt;&gt;"")+--(I11&lt;&gt;"")+--(J11&lt;&gt;"")+--(K11&lt;&gt;"")+--(L11&lt;&gt;"")+--(M11&lt;&gt;"")+--(N11&lt;&gt;"")+--(O11&lt;&gt;"")+--(P11&lt;&gt;"")+--(Q11&lt;&gt;"")+--(R11&lt;&gt;"")+--(S11&lt;&gt;"")+--(T11&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA11" s="16" t="n"/>
-      <c r="AB11" s="16" t="n"/>
-      <c r="AC11" s="16" t="n"/>
-      <c r="AD11" s="16" t="n"/>
+      <c r="AA11" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AB11" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AC11" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="AD11" s="18" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
       <c r="AE11" s="7">
         <f>IF(B11="","",IF(AND(AA11="合格",AB11="合格",AC11="合格",AD11="合格"),"有效","无效"))</f>
         <v/>
@@ -27438,229 +28464,817 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="15">
         <f>IF(B2="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B2" s="16" t="n"/>
-      <c r="C2" s="17" t="n"/>
-      <c r="D2" s="16" t="n"/>
-      <c r="E2" s="16" t="n"/>
-      <c r="F2" s="16" t="n"/>
-      <c r="G2" s="16" t="n"/>
-      <c r="H2" s="16" t="n"/>
-      <c r="I2" s="16" t="n"/>
-      <c r="J2" s="18" t="n"/>
-      <c r="K2" s="16" t="n"/>
-      <c r="L2" s="17" t="n"/>
-      <c r="M2" s="18" t="n"/>
-      <c r="N2" s="16" t="n"/>
-      <c r="O2" s="16" t="n"/>
-      <c r="P2" s="16" t="n"/>
-      <c r="Q2" s="16" t="n"/>
-      <c r="R2" s="16" t="n"/>
-      <c r="S2" s="16" t="n"/>
-      <c r="T2" s="18" t="n"/>
-      <c r="U2" s="18" t="n"/>
-      <c r="V2" s="7">
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>20250626-001</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="n">
+        <v>45834</v>
+      </c>
+      <c r="D2" s="18" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="E2" s="18" t="inlineStr">
+        <is>
+          <t>前高</t>
+        </is>
+      </c>
+      <c r="F2" s="18" t="inlineStr">
+        <is>
+          <t>33.30-33.40</t>
+        </is>
+      </c>
+      <c r="G2" s="18" t="inlineStr">
+        <is>
+          <t>冲高回落</t>
+        </is>
+      </c>
+      <c r="H2" s="18" t="inlineStr">
+        <is>
+          <t>高位分歧</t>
+        </is>
+      </c>
+      <c r="I2" s="18" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="J2" s="18" t="inlineStr">
+        <is>
+          <t>后续只看是否收盘重新站上33.40。</t>
+        </is>
+      </c>
+      <c r="K2" s="18" t="inlineStr">
+        <is>
+          <t>3日</t>
+        </is>
+      </c>
+      <c r="L2" s="28" t="n">
+        <v>45839</v>
+      </c>
+      <c r="M2" s="18" t="inlineStr">
+        <is>
+          <t>收33.97，盘中34.38，已重新站上33.40但没有收过34.08。</t>
+        </is>
+      </c>
+      <c r="N2" s="18" t="inlineStr">
+        <is>
+          <t>向上延续</t>
+        </is>
+      </c>
+      <c r="O2" s="18" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="P2" s="18" t="inlineStr">
+        <is>
+          <t>出现</t>
+        </is>
+      </c>
+      <c r="Q2" s="18" t="inlineStr">
+        <is>
+          <t>削弱</t>
+        </is>
+      </c>
+      <c r="R2" s="18" t="inlineStr">
+        <is>
+          <t>过程合理</t>
+        </is>
+      </c>
+      <c r="S2" s="18" t="inlineStr">
+        <is>
+          <t>概率结果失败</t>
+        </is>
+      </c>
+      <c r="T2" s="18" t="inlineStr">
+        <is>
+          <t>前高分歧不等于失败，必须等收盘确认。</t>
+        </is>
+      </c>
+      <c r="U2" s="18" t="inlineStr">
+        <is>
+          <t>收盘确认与盘中突破区别</t>
+        </is>
+      </c>
+      <c r="V2" s="29">
         <f>IF(L2="","",IF(TODAY()&gt;=L2,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W2" s="16" t="n"/>
-      <c r="X2" s="16" t="n"/>
-    </row>
-    <row r="3">
+      <c r="W2" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="X2" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="72" customHeight="1">
       <c r="A3" s="15">
         <f>IF(B3="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B3" s="16" t="n"/>
-      <c r="C3" s="17" t="n"/>
-      <c r="D3" s="16" t="n"/>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="16" t="n"/>
-      <c r="G3" s="16" t="n"/>
-      <c r="H3" s="16" t="n"/>
-      <c r="I3" s="16" t="n"/>
-      <c r="J3" s="18" t="n"/>
-      <c r="K3" s="16" t="n"/>
-      <c r="L3" s="17" t="n"/>
-      <c r="M3" s="18" t="n"/>
-      <c r="N3" s="16" t="n"/>
-      <c r="O3" s="16" t="n"/>
-      <c r="P3" s="16" t="n"/>
-      <c r="Q3" s="16" t="n"/>
-      <c r="R3" s="16" t="n"/>
-      <c r="S3" s="16" t="n"/>
-      <c r="T3" s="18" t="n"/>
-      <c r="U3" s="18" t="n"/>
-      <c r="V3" s="7">
+      <c r="B3" s="18" t="inlineStr">
+        <is>
+          <t>20250627-002</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="n">
+        <v>45835</v>
+      </c>
+      <c r="D3" s="18" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="E3" s="18" t="inlineStr">
+        <is>
+          <t>前高</t>
+        </is>
+      </c>
+      <c r="F3" s="18" t="inlineStr">
+        <is>
+          <t>33.40</t>
+        </is>
+      </c>
+      <c r="G3" s="18" t="inlineStr">
+        <is>
+          <t>放量突破</t>
+        </is>
+      </c>
+      <c r="H3" s="18" t="inlineStr">
+        <is>
+          <t>真突破/启动尝试</t>
+        </is>
+      </c>
+      <c r="I3" s="18" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="J3" s="18" t="inlineStr">
+        <is>
+          <t>后续只看是否守住33.30-33.40。</t>
+        </is>
+      </c>
+      <c r="K3" s="18" t="inlineStr">
+        <is>
+          <t>3日</t>
+        </is>
+      </c>
+      <c r="L3" s="28" t="n">
+        <v>45840</v>
+      </c>
+      <c r="M3" s="18" t="inlineStr">
+        <is>
+          <t>收33.31，基本回踩到33.30附近，未明显跌破但突破延续不足。</t>
+        </is>
+      </c>
+      <c r="N3" s="18" t="inlineStr">
+        <is>
+          <t>震荡消化</t>
+        </is>
+      </c>
+      <c r="O3" s="18" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="P3" s="18" t="inlineStr">
+        <is>
+          <t>部分出现</t>
+        </is>
+      </c>
+      <c r="Q3" s="18" t="inlineStr">
+        <is>
+          <t>削弱</t>
+        </is>
+      </c>
+      <c r="R3" s="18" t="inlineStr">
+        <is>
+          <t>过程合理</t>
+        </is>
+      </c>
+      <c r="S3" s="18" t="inlineStr">
+        <is>
+          <t>无明显错误</t>
+        </is>
+      </c>
+      <c r="T3" s="18" t="inlineStr">
+        <is>
+          <t>突破后如果不能继续放量，先按震荡消化处理。</t>
+        </is>
+      </c>
+      <c r="U3" s="18" t="inlineStr">
+        <is>
+          <t>突破后的回踩确认</t>
+        </is>
+      </c>
+      <c r="V3" s="29">
         <f>IF(L3="","",IF(TODAY()&gt;=L3,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W3" s="16" t="n"/>
-      <c r="X3" s="16" t="n"/>
-    </row>
-    <row r="4">
+      <c r="W3" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="X3" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="72" customHeight="1">
       <c r="A4" s="15">
         <f>IF(B4="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="17" t="n"/>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="16" t="n"/>
-      <c r="G4" s="16" t="n"/>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="16" t="n"/>
-      <c r="J4" s="18" t="n"/>
-      <c r="K4" s="16" t="n"/>
-      <c r="L4" s="17" t="n"/>
-      <c r="M4" s="18" t="n"/>
-      <c r="N4" s="16" t="n"/>
-      <c r="O4" s="16" t="n"/>
-      <c r="P4" s="16" t="n"/>
-      <c r="Q4" s="16" t="n"/>
-      <c r="R4" s="16" t="n"/>
-      <c r="S4" s="16" t="n"/>
-      <c r="T4" s="18" t="n"/>
-      <c r="U4" s="18" t="n"/>
-      <c r="V4" s="7">
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>20250630-003</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="n">
+        <v>45838</v>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>前高</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>34.08</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>横盘震荡</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>震荡整理</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>后续只看是否收盘站上34.08。</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>3日</t>
+        </is>
+      </c>
+      <c r="L4" s="28" t="n">
+        <v>45841</v>
+      </c>
+      <c r="M4" s="18" t="inlineStr">
+        <is>
+          <t>收33.53，未站上34.08，仍在33.20-34.08之间。</t>
+        </is>
+      </c>
+      <c r="N4" s="18" t="inlineStr">
+        <is>
+          <t>震荡消化</t>
+        </is>
+      </c>
+      <c r="O4" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="P4" s="18" t="inlineStr">
+        <is>
+          <t>未出现</t>
+        </is>
+      </c>
+      <c r="Q4" s="18" t="inlineStr">
+        <is>
+          <t>强化</t>
+        </is>
+      </c>
+      <c r="R4" s="18" t="inlineStr">
+        <is>
+          <t>过程合理</t>
+        </is>
+      </c>
+      <c r="S4" s="18" t="inlineStr">
+        <is>
+          <t>无明显错误</t>
+        </is>
+      </c>
+      <c r="T4" s="18" t="inlineStr">
+        <is>
+          <t>低强度震荡判断可以接受，不需要硬预测方向。</t>
+        </is>
+      </c>
+      <c r="U4" s="18" t="inlineStr">
+        <is>
+          <t>箱体上沿确认</t>
+        </is>
+      </c>
+      <c r="V4" s="29">
         <f>IF(L4="","",IF(TODAY()&gt;=L4,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W4" s="16" t="n"/>
-      <c r="X4" s="16" t="n"/>
-    </row>
-    <row r="5">
+      <c r="W4" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="X4" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="15">
         <f>IF(B5="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B5" s="16" t="n"/>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
-      <c r="J5" s="18" t="n"/>
-      <c r="K5" s="16" t="n"/>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="18" t="n"/>
-      <c r="N5" s="16" t="n"/>
-      <c r="O5" s="16" t="n"/>
-      <c r="P5" s="16" t="n"/>
-      <c r="Q5" s="16" t="n"/>
-      <c r="R5" s="16" t="n"/>
-      <c r="S5" s="16" t="n"/>
-      <c r="T5" s="18" t="n"/>
-      <c r="U5" s="18" t="n"/>
-      <c r="V5" s="7">
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>20250701-004</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="n">
+        <v>45839</v>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>前高</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>34.08</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>高位放量震荡</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>高位分歧</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>后续只看是否收盘站上34.08。</t>
+        </is>
+      </c>
+      <c r="K5" s="18" t="inlineStr">
+        <is>
+          <t>3日</t>
+        </is>
+      </c>
+      <c r="L5" s="28" t="n">
+        <v>45842</v>
+      </c>
+      <c r="M5" s="18" t="inlineStr">
+        <is>
+          <t>收33.23，没有站回34.08，反而回到短线下沿。</t>
+        </is>
+      </c>
+      <c r="N5" s="18" t="inlineStr">
+        <is>
+          <t>冲高回落</t>
+        </is>
+      </c>
+      <c r="O5" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="P5" s="18" t="inlineStr">
+        <is>
+          <t>未出现</t>
+        </is>
+      </c>
+      <c r="Q5" s="18" t="inlineStr">
+        <is>
+          <t>强化</t>
+        </is>
+      </c>
+      <c r="R5" s="18" t="inlineStr">
+        <is>
+          <t>过程合理</t>
+        </is>
+      </c>
+      <c r="S5" s="18" t="inlineStr">
+        <is>
+          <t>无明显错误</t>
+        </is>
+      </c>
+      <c r="T5" s="18" t="inlineStr">
+        <is>
+          <t>盘中新高不如收盘站稳重要。</t>
+        </is>
+      </c>
+      <c r="U5" s="18" t="inlineStr">
+        <is>
+          <t>假突破与分歧换手区分</t>
+        </is>
+      </c>
+      <c r="V5" s="29">
         <f>IF(L5="","",IF(TODAY()&gt;=L5,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W5" s="16" t="n"/>
-      <c r="X5" s="16" t="n"/>
-    </row>
-    <row r="6">
+      <c r="W5" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="X5" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
       <c r="A6" s="15">
         <f>IF(B6="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="16" t="n"/>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="16" t="n"/>
-      <c r="G6" s="16" t="n"/>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="16" t="n"/>
-      <c r="J6" s="18" t="n"/>
-      <c r="K6" s="16" t="n"/>
-      <c r="L6" s="17" t="n"/>
-      <c r="M6" s="18" t="n"/>
-      <c r="N6" s="16" t="n"/>
-      <c r="O6" s="16" t="n"/>
-      <c r="P6" s="16" t="n"/>
-      <c r="Q6" s="16" t="n"/>
-      <c r="R6" s="16" t="n"/>
-      <c r="S6" s="16" t="n"/>
-      <c r="T6" s="18" t="n"/>
-      <c r="U6" s="18" t="n"/>
-      <c r="V6" s="7">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>20250702-005</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n">
+        <v>45840</v>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>大阳线低点</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>33.00-33.30</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>缩量回调</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>健康回调</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>后续只看是否跌破33.00。</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>3日</t>
+        </is>
+      </c>
+      <c r="L6" s="28" t="n">
+        <v>45845</v>
+      </c>
+      <c r="M6" s="18" t="inlineStr">
+        <is>
+          <t>收32.95，跌破33.00，但成交量继续缩小。</t>
+        </is>
+      </c>
+      <c r="N6" s="18" t="inlineStr">
+        <is>
+          <t>跌破支撑</t>
+        </is>
+      </c>
+      <c r="O6" s="18" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="P6" s="18" t="inlineStr">
+        <is>
+          <t>出现</t>
+        </is>
+      </c>
+      <c r="Q6" s="18" t="inlineStr">
+        <is>
+          <t>证伪</t>
+        </is>
+      </c>
+      <c r="R6" s="18" t="inlineStr">
+        <is>
+          <t>概率失败</t>
+        </is>
+      </c>
+      <c r="S6" s="18" t="inlineStr">
+        <is>
+          <t>概率结果失败</t>
+        </is>
+      </c>
+      <c r="T6" s="18" t="inlineStr">
+        <is>
+          <t>健康回调假设被证伪时要切换解释，不要补理由。</t>
+        </is>
+      </c>
+      <c r="U6" s="18" t="inlineStr">
+        <is>
+          <t>支撑区间有效性</t>
+        </is>
+      </c>
+      <c r="V6" s="29">
         <f>IF(L6="","",IF(TODAY()&gt;=L6,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W6" s="16" t="n"/>
-      <c r="X6" s="16" t="n"/>
-    </row>
-    <row r="7">
+      <c r="W6" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="X6" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
       <c r="A7" s="15">
         <f>IF(B7="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
-      <c r="J7" s="18" t="n"/>
-      <c r="K7" s="16" t="n"/>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="18" t="n"/>
-      <c r="N7" s="16" t="n"/>
-      <c r="O7" s="16" t="n"/>
-      <c r="P7" s="16" t="n"/>
-      <c r="Q7" s="16" t="n"/>
-      <c r="R7" s="16" t="n"/>
-      <c r="S7" s="16" t="n"/>
-      <c r="T7" s="18" t="n"/>
-      <c r="U7" s="18" t="n"/>
-      <c r="V7" s="7">
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>20250703-006</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="n">
+        <v>45841</v>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>箱体下沿</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>33.20-33.30</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>回踩支撑不破</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>震荡整理</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="J7" s="18" t="inlineStr">
+        <is>
+          <t>后续只看是否跌破33.20。</t>
+        </is>
+      </c>
+      <c r="K7" s="18" t="inlineStr">
+        <is>
+          <t>3日</t>
+        </is>
+      </c>
+      <c r="L7" s="28" t="n">
+        <v>45846</v>
+      </c>
+      <c r="M7" s="18" t="inlineStr">
+        <is>
+          <t>收33.55，未跌破33.20，并重新收回33.40上方。</t>
+        </is>
+      </c>
+      <c r="N7" s="18" t="inlineStr">
+        <is>
+          <t>修复转强</t>
+        </is>
+      </c>
+      <c r="O7" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="P7" s="18" t="inlineStr">
+        <is>
+          <t>未出现</t>
+        </is>
+      </c>
+      <c r="Q7" s="18" t="inlineStr">
+        <is>
+          <t>强化</t>
+        </is>
+      </c>
+      <c r="R7" s="18" t="inlineStr">
+        <is>
+          <t>过程合理</t>
+        </is>
+      </c>
+      <c r="S7" s="18" t="inlineStr">
+        <is>
+          <t>无明显错误</t>
+        </is>
+      </c>
+      <c r="T7" s="18" t="inlineStr">
+        <is>
+          <t>两个低点形成的临时箱体可以观察，但强度要低。</t>
+        </is>
+      </c>
+      <c r="U7" s="18" t="inlineStr">
+        <is>
+          <t>临时箱体识别</t>
+        </is>
+      </c>
+      <c r="V7" s="29">
         <f>IF(L7="","",IF(TODAY()&gt;=L7,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W7" s="16" t="n"/>
-      <c r="X7" s="16" t="n"/>
-    </row>
-    <row r="8">
+      <c r="W7" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="X7" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
       <c r="A8" s="15">
         <f>IF(B8="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="17" t="n"/>
-      <c r="D8" s="16" t="n"/>
-      <c r="E8" s="16" t="n"/>
-      <c r="F8" s="16" t="n"/>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="16" t="n"/>
-      <c r="J8" s="18" t="n"/>
-      <c r="K8" s="16" t="n"/>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="18" t="n"/>
-      <c r="N8" s="16" t="n"/>
-      <c r="O8" s="16" t="n"/>
-      <c r="P8" s="16" t="n"/>
-      <c r="Q8" s="16" t="n"/>
-      <c r="R8" s="16" t="n"/>
-      <c r="S8" s="16" t="n"/>
-      <c r="T8" s="18" t="n"/>
-      <c r="U8" s="18" t="n"/>
-      <c r="V8" s="7">
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>20250704-007</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="n">
+        <v>45842</v>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>长电科技 600584.SH</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>箱体下沿</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>33.20-33.30</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>横盘震荡</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>震荡整理</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>后续只看是否跌破33.00。</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>3日</t>
+        </is>
+      </c>
+      <c r="L8" s="28" t="n">
+        <v>45847</v>
+      </c>
+      <c r="M8" s="18" t="inlineStr">
+        <is>
+          <t>收33.18，未跌破33.00，但也没有向上确认。</t>
+        </is>
+      </c>
+      <c r="N8" s="18" t="inlineStr">
+        <is>
+          <t>震荡消化</t>
+        </is>
+      </c>
+      <c r="O8" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="P8" s="18" t="inlineStr">
+        <is>
+          <t>未出现</t>
+        </is>
+      </c>
+      <c r="Q8" s="18" t="inlineStr">
+        <is>
+          <t>仍不确定</t>
+        </is>
+      </c>
+      <c r="R8" s="18" t="inlineStr">
+        <is>
+          <t>过程合理</t>
+        </is>
+      </c>
+      <c r="S8" s="18" t="inlineStr">
+        <is>
+          <t>无明显错误</t>
+        </is>
+      </c>
+      <c r="T8" s="18" t="inlineStr">
+        <is>
+          <t>低强度判断允许保持不确定，不必强行改成看多或看空。</t>
+        </is>
+      </c>
+      <c r="U8" s="18" t="inlineStr">
+        <is>
+          <t>方向不明时的观察纪律</t>
+        </is>
+      </c>
+      <c r="V8" s="29">
         <f>IF(L8="","",IF(TODAY()&gt;=L8,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W8" s="16" t="n"/>
-      <c r="X8" s="16" t="n"/>
+      <c r="W8" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="X8" s="18" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="15">
@@ -43472,6 +45086,8 @@
           <t>训练看板</t>
         </is>
       </c>
+      <c r="B1" s="22" t="n"/>
+      <c r="C1" s="23" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -43792,7 +45408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -44500,7 +46116,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Clear stock template sample data
</commit_message>
<xml_diff>
--- a/stock_review_template.xlsx
+++ b/stock_review_template.xlsx
@@ -794,32 +794,16 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="24" t="inlineStr">
-        <is>
-          <t>长电科技10日样本数据说明</t>
-        </is>
-      </c>
+      <c r="A28" s="24" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="24" t="inlineStr">
-        <is>
-          <t>样本写入位置：每日观察!2:11，事后验证!2:8。</t>
-        </is>
-      </c>
+      <c r="A29" s="24" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="24" t="inlineStr">
-        <is>
-          <t>个股数据：搜狐历史行情接口 cn_600584；大盘数据：搜狐历史行情接口 zs_000001；板块数据：东方财富半导体板块 BK1036。</t>
-        </is>
-      </c>
+      <c r="A30" s="24" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="24" t="inlineStr">
-        <is>
-          <t>样本日期范围：2025-06-26 至 2025-07-09，共10个交易日；因当前接口未返回2026年数据，本样本按可取得的最近完整窗口填写。</t>
-        </is>
-      </c>
+      <c r="A31" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1028,114 +1012,32 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="72" customHeight="1">
+    <row r="2">
       <c r="A2" s="7">
         <f>IF(B2="","",TEXT(B2,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B2" s="25" t="n">
-        <v>45834</v>
-      </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="D2" s="10" t="inlineStr">
-        <is>
-          <t>半导体/封测</t>
-        </is>
-      </c>
-      <c r="E2" s="10" t="inlineStr">
-        <is>
-          <t>震荡偏强</t>
-        </is>
-      </c>
-      <c r="F2" s="10" t="inlineStr">
-        <is>
-          <t>震荡</t>
-        </is>
-      </c>
-      <c r="G2" s="10" t="inlineStr">
-        <is>
-          <t>强于板块</t>
-        </is>
-      </c>
-      <c r="H2" s="10" t="inlineStr">
-        <is>
-          <t>前高</t>
-        </is>
-      </c>
-      <c r="I2" s="10" t="inlineStr">
-        <is>
-          <t>33.30-33.40</t>
-        </is>
-      </c>
-      <c r="J2" s="10" t="inlineStr">
-        <is>
-          <t>6月25日前高33.30，今日最高33.40但收32.96，说明上方第一次出现分歧。</t>
-        </is>
-      </c>
-      <c r="K2" s="10" t="inlineStr">
-        <is>
-          <t>接近</t>
-        </is>
-      </c>
-      <c r="L2" s="10" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="M2" s="10" t="inlineStr">
-        <is>
-          <t>冲高回落</t>
-        </is>
-      </c>
-      <c r="N2" s="10" t="inlineStr">
-        <is>
-          <t>收32.96跌0.78%，盘中最高33.40触及前高区，成交量26.21万手；半导体跌1.17%，上证跌0.22%。</t>
-        </is>
-      </c>
-      <c r="O2" s="10" t="inlineStr">
-        <is>
-          <t>高位分歧</t>
-        </is>
-      </c>
-      <c r="P2" s="10" t="inlineStr">
-        <is>
-          <t>价格接近前高后没有收住，说明33.30-33.40附近存在短线抛压；但个股跌幅小于半导体，不能直接判定转弱。</t>
-        </is>
-      </c>
-      <c r="Q2" s="10" t="inlineStr">
-        <is>
-          <t>如果随后1-3日重新放量站上33.40，今天更像突破前正常分歧，而不是上攻失败。</t>
-        </is>
-      </c>
-      <c r="R2" s="10" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="S2" s="10" t="inlineStr">
-        <is>
-          <t>有明确前高和冲高回落事实，但板块当天较弱，单日不能确认失败。</t>
-        </is>
-      </c>
-      <c r="T2" s="10" t="inlineStr">
-        <is>
-          <t>后续只看是否收盘重新站上33.40。</t>
-        </is>
-      </c>
-      <c r="U2" s="11" t="inlineStr">
-        <is>
-          <t>前高区间确认、冲高回落与板块环境区分</t>
-        </is>
-      </c>
-      <c r="V2" s="11" t="inlineStr">
-        <is>
-          <t>数据源：搜狐历史行情个股；东方财富半导体板块；窗口为2025-06-26至2025-07-09。</t>
-        </is>
-      </c>
+      <c r="B2" s="25" t="n"/>
+      <c r="C2" s="10" t="n"/>
+      <c r="D2" s="10" t="n"/>
+      <c r="E2" s="10" t="n"/>
+      <c r="F2" s="10" t="n"/>
+      <c r="G2" s="10" t="n"/>
+      <c r="H2" s="10" t="n"/>
+      <c r="I2" s="10" t="n"/>
+      <c r="J2" s="10" t="n"/>
+      <c r="K2" s="10" t="n"/>
+      <c r="L2" s="10" t="n"/>
+      <c r="M2" s="10" t="n"/>
+      <c r="N2" s="10" t="n"/>
+      <c r="O2" s="10" t="n"/>
+      <c r="P2" s="10" t="n"/>
+      <c r="Q2" s="10" t="n"/>
+      <c r="R2" s="10" t="n"/>
+      <c r="S2" s="10" t="n"/>
+      <c r="T2" s="10" t="n"/>
+      <c r="U2" s="11" t="n"/>
+      <c r="V2" s="11" t="n"/>
       <c r="W2" s="26">
         <f>IF(B2="","",B2+3)</f>
         <v/>
@@ -1152,139 +1054,41 @@
         <f>IF(B2="","",(--(B2&lt;&gt;"")+--(C2&lt;&gt;"")+--(D2&lt;&gt;"")+--(E2&lt;&gt;"")+--(F2&lt;&gt;"")+--(G2&lt;&gt;"")+--(H2&lt;&gt;"")+--(I2&lt;&gt;"")+--(J2&lt;&gt;"")+--(K2&lt;&gt;"")+--(L2&lt;&gt;"")+--(M2&lt;&gt;"")+--(N2&lt;&gt;"")+--(O2&lt;&gt;"")+--(P2&lt;&gt;"")+--(Q2&lt;&gt;"")+--(R2&lt;&gt;"")+--(S2&lt;&gt;"")+--(T2&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA2" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AB2" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AC2" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AD2" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
+      <c r="AA2" s="18" t="n"/>
+      <c r="AB2" s="18" t="n"/>
+      <c r="AC2" s="18" t="n"/>
+      <c r="AD2" s="18" t="n"/>
       <c r="AE2" s="7">
         <f>IF(B2="","",IF(AND(AA2="合格",AB2="合格",AC2="合格",AD2="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="3" ht="72" customHeight="1">
+    <row r="3">
       <c r="A3" s="7">
         <f>IF(B3="","",TEXT(B3,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B3" s="25" t="n">
-        <v>45835</v>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>半导体/封测</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>震荡</t>
-        </is>
-      </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>轮动强势</t>
-        </is>
-      </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>强于板块</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
-        <is>
-          <t>前高</t>
-        </is>
-      </c>
-      <c r="I3" s="10" t="inlineStr">
-        <is>
-          <t>33.40</t>
-        </is>
-      </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>前一日最高33.40形成短线压力，今日最高34.08且收33.60。</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>突破</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>清晰</t>
-        </is>
-      </c>
-      <c r="M3" s="10" t="inlineStr">
-        <is>
-          <t>放量突破</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>收33.60涨1.94%，最高34.08，成交量46.41万手明显放大；半导体涨1.08%，上证跌0.70%。</t>
-        </is>
-      </c>
-      <c r="O3" s="10" t="inlineStr">
-        <is>
-          <t>真突破/启动尝试</t>
-        </is>
-      </c>
-      <c r="P3" s="10" t="inlineStr">
-        <is>
-          <t>在大盘走弱时个股放量收过33.40，且强于半导体，说明有资金主动推动突破。</t>
-        </is>
-      </c>
-      <c r="Q3" s="10" t="inlineStr">
-        <is>
-          <t>收盘离日高较远，若很快跌回33.40下方并放量，突破解释会削弱。</t>
-        </is>
-      </c>
-      <c r="R3" s="10" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="S3" s="10" t="inlineStr">
-        <is>
-          <t>量价与相对强弱都支持，但只是一日突破，还没有回踩确认。</t>
-        </is>
-      </c>
-      <c r="T3" s="10" t="inlineStr">
-        <is>
-          <t>后续只看是否守住33.30-33.40。</t>
-        </is>
-      </c>
-      <c r="U3" s="11" t="inlineStr">
-        <is>
-          <t>突破有效性、放量含义、回踩确认</t>
-        </is>
-      </c>
-      <c r="V3" s="11" t="inlineStr">
-        <is>
-          <t>这是突破尝试，不等于已经进入主升。</t>
-        </is>
-      </c>
+      <c r="B3" s="25" t="n"/>
+      <c r="C3" s="10" t="n"/>
+      <c r="D3" s="10" t="n"/>
+      <c r="E3" s="10" t="n"/>
+      <c r="F3" s="10" t="n"/>
+      <c r="G3" s="10" t="n"/>
+      <c r="H3" s="10" t="n"/>
+      <c r="I3" s="10" t="n"/>
+      <c r="J3" s="10" t="n"/>
+      <c r="K3" s="10" t="n"/>
+      <c r="L3" s="10" t="n"/>
+      <c r="M3" s="10" t="n"/>
+      <c r="N3" s="10" t="n"/>
+      <c r="O3" s="10" t="n"/>
+      <c r="P3" s="10" t="n"/>
+      <c r="Q3" s="10" t="n"/>
+      <c r="R3" s="10" t="n"/>
+      <c r="S3" s="10" t="n"/>
+      <c r="T3" s="10" t="n"/>
+      <c r="U3" s="11" t="n"/>
+      <c r="V3" s="11" t="n"/>
       <c r="W3" s="26">
         <f>IF(B3="","",B3+3)</f>
         <v/>
@@ -1301,139 +1105,41 @@
         <f>IF(B3="","",(--(B3&lt;&gt;"")+--(C3&lt;&gt;"")+--(D3&lt;&gt;"")+--(E3&lt;&gt;"")+--(F3&lt;&gt;"")+--(G3&lt;&gt;"")+--(H3&lt;&gt;"")+--(I3&lt;&gt;"")+--(J3&lt;&gt;"")+--(K3&lt;&gt;"")+--(L3&lt;&gt;"")+--(M3&lt;&gt;"")+--(N3&lt;&gt;"")+--(O3&lt;&gt;"")+--(P3&lt;&gt;"")+--(Q3&lt;&gt;"")+--(R3&lt;&gt;"")+--(S3&lt;&gt;"")+--(T3&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA3" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AB3" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AC3" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AD3" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
+      <c r="AA3" s="18" t="n"/>
+      <c r="AB3" s="18" t="n"/>
+      <c r="AC3" s="18" t="n"/>
+      <c r="AD3" s="18" t="n"/>
       <c r="AE3" s="7">
         <f>IF(B3="","",IF(AND(AA3="合格",AB3="合格",AC3="合格",AD3="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="4" ht="72" customHeight="1">
+    <row r="4">
       <c r="A4" s="7">
         <f>IF(B4="","",TEXT(B4,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B4" s="25" t="n">
-        <v>45838</v>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>半导体/封测</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>震荡偏强</t>
-        </is>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>主线强势</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>弱于板块</t>
-        </is>
-      </c>
-      <c r="H4" s="10" t="inlineStr">
-        <is>
-          <t>前高</t>
-        </is>
-      </c>
-      <c r="I4" s="10" t="inlineStr">
-        <is>
-          <t>34.08</t>
-        </is>
-      </c>
-      <c r="J4" s="10" t="inlineStr">
-        <is>
-          <t>6月27日突破日最高34.08是新的短线观察压力。</t>
-        </is>
-      </c>
-      <c r="K4" s="10" t="inlineStr">
-        <is>
-          <t>接近</t>
-        </is>
-      </c>
-      <c r="L4" s="10" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="M4" s="10" t="inlineStr">
-        <is>
-          <t>横盘震荡</t>
-        </is>
-      </c>
-      <c r="N4" s="10" t="inlineStr">
-        <is>
-          <t>收33.69涨0.27%，成交量30.02万手缩小；半导体涨1.67%，上证涨0.59%。</t>
-        </is>
-      </c>
-      <c r="O4" s="10" t="inlineStr">
-        <is>
-          <t>震荡整理</t>
-        </is>
-      </c>
-      <c r="P4" s="10" t="inlineStr">
-        <is>
-          <t>突破后没有继续放量上攻，只是在33.40上方小幅整理；但弱于强势板块，说明主动性不足。</t>
-        </is>
-      </c>
-      <c r="Q4" s="10" t="inlineStr">
-        <is>
-          <t>如果次日放量站上34.08，则今天的缩量可能只是突破后的蓄势。</t>
-        </is>
-      </c>
-      <c r="R4" s="10" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="S4" s="10" t="inlineStr">
-        <is>
-          <t>事实更多指向整理，但是否转弱还缺少跌破关键位。</t>
-        </is>
-      </c>
-      <c r="T4" s="10" t="inlineStr">
-        <is>
-          <t>后续只看是否收盘站上34.08。</t>
-        </is>
-      </c>
-      <c r="U4" s="11" t="inlineStr">
-        <is>
-          <t>突破后缩量整理、相对板块弱势识别</t>
-        </is>
-      </c>
-      <c r="V4" s="11" t="inlineStr">
-        <is>
-          <t>这一天的重点不是预测涨跌，而是识别“突破后没有立刻延续”。</t>
-        </is>
-      </c>
+      <c r="B4" s="25" t="n"/>
+      <c r="C4" s="10" t="n"/>
+      <c r="D4" s="10" t="n"/>
+      <c r="E4" s="10" t="n"/>
+      <c r="F4" s="10" t="n"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="10" t="n"/>
+      <c r="I4" s="10" t="n"/>
+      <c r="J4" s="10" t="n"/>
+      <c r="K4" s="10" t="n"/>
+      <c r="L4" s="10" t="n"/>
+      <c r="M4" s="10" t="n"/>
+      <c r="N4" s="10" t="n"/>
+      <c r="O4" s="10" t="n"/>
+      <c r="P4" s="10" t="n"/>
+      <c r="Q4" s="10" t="n"/>
+      <c r="R4" s="10" t="n"/>
+      <c r="S4" s="10" t="n"/>
+      <c r="T4" s="10" t="n"/>
+      <c r="U4" s="11" t="n"/>
+      <c r="V4" s="11" t="n"/>
       <c r="W4" s="26">
         <f>IF(B4="","",B4+3)</f>
         <v/>
@@ -1450,139 +1156,41 @@
         <f>IF(B4="","",(--(B4&lt;&gt;"")+--(C4&lt;&gt;"")+--(D4&lt;&gt;"")+--(E4&lt;&gt;"")+--(F4&lt;&gt;"")+--(G4&lt;&gt;"")+--(H4&lt;&gt;"")+--(I4&lt;&gt;"")+--(J4&lt;&gt;"")+--(K4&lt;&gt;"")+--(L4&lt;&gt;"")+--(M4&lt;&gt;"")+--(N4&lt;&gt;"")+--(O4&lt;&gt;"")+--(P4&lt;&gt;"")+--(Q4&lt;&gt;"")+--(R4&lt;&gt;"")+--(S4&lt;&gt;"")+--(T4&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA4" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AB4" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AC4" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AD4" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
+      <c r="AA4" s="18" t="n"/>
+      <c r="AB4" s="18" t="n"/>
+      <c r="AC4" s="18" t="n"/>
+      <c r="AD4" s="18" t="n"/>
       <c r="AE4" s="7">
         <f>IF(B4="","",IF(AND(AA4="合格",AB4="合格",AC4="合格",AD4="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="5" ht="72" customHeight="1">
+    <row r="5">
       <c r="A5" s="7">
         <f>IF(B5="","",TEXT(B5,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B5" s="25" t="n">
-        <v>45839</v>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>半导体/封测</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>震荡偏强</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>轮动强势</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>强于板块</t>
-        </is>
-      </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>前高</t>
-        </is>
-      </c>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>34.08</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>6月27日高点34.08被盘中突破，但收盘33.97没有站上。</t>
-        </is>
-      </c>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>站上未确认</t>
-        </is>
-      </c>
-      <c r="L5" s="10" t="inlineStr">
-        <is>
-          <t>清晰</t>
-        </is>
-      </c>
-      <c r="M5" s="10" t="inlineStr">
-        <is>
-          <t>高位放量震荡</t>
-        </is>
-      </c>
-      <c r="N5" s="10" t="inlineStr">
-        <is>
-          <t>收33.97涨0.83%，盘中最高34.38创短线新高，成交量39.29万手；半导体涨0.33%，上证涨0.39%。</t>
-        </is>
-      </c>
-      <c r="O5" s="10" t="inlineStr">
-        <is>
-          <t>高位分歧</t>
-        </is>
-      </c>
-      <c r="P5" s="10" t="inlineStr">
-        <is>
-          <t>盘中新高但收回34.08下方，说明新高位置有抛压；不过个股仍强于板块，不能直接判定见顶。</t>
-        </is>
-      </c>
-      <c r="Q5" s="10" t="inlineStr">
-        <is>
-          <t>如果后续收盘站回34.08并继续放量，新高回落可能只是分歧换手。</t>
-        </is>
-      </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="S5" s="10" t="inlineStr">
-        <is>
-          <t>关键位清晰且有冲高回落，但趋势尚未破坏。</t>
-        </is>
-      </c>
-      <c r="T5" s="10" t="inlineStr">
-        <is>
-          <t>后续只看是否收盘站上34.08。</t>
-        </is>
-      </c>
-      <c r="U5" s="11" t="inlineStr">
-        <is>
-          <t>盘中新高与收盘确认、分歧换手</t>
-        </is>
-      </c>
-      <c r="V5" s="11" t="inlineStr">
-        <is>
-          <t>这是判断“真突破还是假突破”的典型样本。</t>
-        </is>
-      </c>
+      <c r="B5" s="25" t="n"/>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="10" t="n"/>
+      <c r="H5" s="10" t="n"/>
+      <c r="I5" s="10" t="n"/>
+      <c r="J5" s="10" t="n"/>
+      <c r="K5" s="10" t="n"/>
+      <c r="L5" s="10" t="n"/>
+      <c r="M5" s="10" t="n"/>
+      <c r="N5" s="10" t="n"/>
+      <c r="O5" s="10" t="n"/>
+      <c r="P5" s="10" t="n"/>
+      <c r="Q5" s="10" t="n"/>
+      <c r="R5" s="10" t="n"/>
+      <c r="S5" s="10" t="n"/>
+      <c r="T5" s="10" t="n"/>
+      <c r="U5" s="11" t="n"/>
+      <c r="V5" s="11" t="n"/>
       <c r="W5" s="26">
         <f>IF(B5="","",B5+3)</f>
         <v/>
@@ -1599,139 +1207,41 @@
         <f>IF(B5="","",(--(B5&lt;&gt;"")+--(C5&lt;&gt;"")+--(D5&lt;&gt;"")+--(E5&lt;&gt;"")+--(F5&lt;&gt;"")+--(G5&lt;&gt;"")+--(H5&lt;&gt;"")+--(I5&lt;&gt;"")+--(J5&lt;&gt;"")+--(K5&lt;&gt;"")+--(L5&lt;&gt;"")+--(M5&lt;&gt;"")+--(N5&lt;&gt;"")+--(O5&lt;&gt;"")+--(P5&lt;&gt;"")+--(Q5&lt;&gt;"")+--(R5&lt;&gt;"")+--(S5&lt;&gt;"")+--(T5&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA5" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AB5" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AC5" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AD5" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
+      <c r="AA5" s="18" t="n"/>
+      <c r="AB5" s="18" t="n"/>
+      <c r="AC5" s="18" t="n"/>
+      <c r="AD5" s="18" t="n"/>
       <c r="AE5" s="7">
         <f>IF(B5="","",IF(AND(AA5="合格",AB5="合格",AC5="合格",AD5="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="6" ht="72" customHeight="1">
+    <row r="6">
       <c r="A6" s="7">
         <f>IF(B6="","",TEXT(B6,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B6" s="25" t="n">
-        <v>45840</v>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>半导体/封测</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>震荡</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>退潮</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>强于板块</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>大阳线低点</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>33.00-33.30</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>6月27日放量阳线低点33.00，6月25日前高33.30附近构成回踩观察区。</t>
-        </is>
-      </c>
-      <c r="K6" s="10" t="inlineStr">
-        <is>
-          <t>回踩</t>
-        </is>
-      </c>
-      <c r="L6" s="10" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="M6" s="10" t="inlineStr">
-        <is>
-          <t>缩量回调</t>
-        </is>
-      </c>
-      <c r="N6" s="10" t="inlineStr">
-        <is>
-          <t>收33.31跌1.94%，最低33.23，成交量26.21万手；半导体跌2.18%，上证跌0.09%。</t>
-        </is>
-      </c>
-      <c r="O6" s="10" t="inlineStr">
-        <is>
-          <t>健康回调</t>
-        </is>
-      </c>
-      <c r="P6" s="10" t="inlineStr">
-        <is>
-          <t>价格回到33.00-33.30支撑区附近但没有明显放量跌破，且跌幅小于半导体，暂时更像突破后的回踩。</t>
-        </is>
-      </c>
-      <c r="Q6" s="10" t="inlineStr">
-        <is>
-          <t>如果随后跌破33.00并收不回，健康回调解释会被证伪。</t>
-        </is>
-      </c>
-      <c r="R6" s="10" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="S6" s="10" t="inlineStr">
-        <is>
-          <t>回踩区间是人工划出来的，不够精确，只能作为低强度假设。</t>
-        </is>
-      </c>
-      <c r="T6" s="10" t="inlineStr">
-        <is>
-          <t>后续只看是否跌破33.00。</t>
-        </is>
-      </c>
-      <c r="U6" s="11" t="inlineStr">
-        <is>
-          <t>大阳线低点、支撑区间而非单点、缩量回调</t>
-        </is>
-      </c>
-      <c r="V6" s="11" t="inlineStr">
-        <is>
-          <t>这行故意保持低判断强度，因为支撑区不是非常清晰。</t>
-        </is>
-      </c>
+      <c r="B6" s="25" t="n"/>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="n"/>
+      <c r="H6" s="10" t="n"/>
+      <c r="I6" s="10" t="n"/>
+      <c r="J6" s="10" t="n"/>
+      <c r="K6" s="10" t="n"/>
+      <c r="L6" s="10" t="n"/>
+      <c r="M6" s="10" t="n"/>
+      <c r="N6" s="10" t="n"/>
+      <c r="O6" s="10" t="n"/>
+      <c r="P6" s="10" t="n"/>
+      <c r="Q6" s="10" t="n"/>
+      <c r="R6" s="10" t="n"/>
+      <c r="S6" s="10" t="n"/>
+      <c r="T6" s="10" t="n"/>
+      <c r="U6" s="11" t="n"/>
+      <c r="V6" s="11" t="n"/>
       <c r="W6" s="26">
         <f>IF(B6="","",B6+3)</f>
         <v/>
@@ -1748,139 +1258,41 @@
         <f>IF(B6="","",(--(B6&lt;&gt;"")+--(C6&lt;&gt;"")+--(D6&lt;&gt;"")+--(E6&lt;&gt;"")+--(F6&lt;&gt;"")+--(G6&lt;&gt;"")+--(H6&lt;&gt;"")+--(I6&lt;&gt;"")+--(J6&lt;&gt;"")+--(K6&lt;&gt;"")+--(L6&lt;&gt;"")+--(M6&lt;&gt;"")+--(N6&lt;&gt;"")+--(O6&lt;&gt;"")+--(P6&lt;&gt;"")+--(Q6&lt;&gt;"")+--(R6&lt;&gt;"")+--(S6&lt;&gt;"")+--(T6&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA6" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AB6" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AC6" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AD6" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
+      <c r="AA6" s="18" t="n"/>
+      <c r="AB6" s="18" t="n"/>
+      <c r="AC6" s="18" t="n"/>
+      <c r="AD6" s="18" t="n"/>
       <c r="AE6" s="7">
         <f>IF(B6="","",IF(AND(AA6="合格",AB6="合格",AC6="合格",AD6="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="7" ht="72" customHeight="1">
+    <row r="7">
       <c r="A7" s="7">
         <f>IF(B7="","",TEXT(B7,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B7" s="25" t="n">
-        <v>45841</v>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>半导体/封测</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>震荡偏强</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>震荡</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>强于板块</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>箱体下沿</t>
-        </is>
-      </c>
-      <c r="I7" s="10" t="inlineStr">
-        <is>
-          <t>33.20-33.30</t>
-        </is>
-      </c>
-      <c r="J7" s="10" t="inlineStr">
-        <is>
-          <t>7月2日低点33.23与7月3日低点33.23重合，形成短线震荡下沿。</t>
-        </is>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
-        <is>
-          <t>回踩</t>
-        </is>
-      </c>
-      <c r="L7" s="10" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="M7" s="10" t="inlineStr">
-        <is>
-          <t>回踩支撑不破</t>
-        </is>
-      </c>
-      <c r="N7" s="10" t="inlineStr">
-        <is>
-          <t>收33.53涨0.66%，最低33.23再次守住，成交量21.32万手继续缩小；半导体涨0.36%，上证涨0.18%。</t>
-        </is>
-      </c>
-      <c r="O7" s="10" t="inlineStr">
-        <is>
-          <t>震荡整理</t>
-        </is>
-      </c>
-      <c r="P7" s="10" t="inlineStr">
-        <is>
-          <t>同一低点附近两次守住，价格没有继续向下；但成交量缩小，说明反弹力度也不强。</t>
-        </is>
-      </c>
-      <c r="Q7" s="10" t="inlineStr">
-        <is>
-          <t>如果后续跌破33.20，所谓箱体下沿就只是临时巧合。</t>
-        </is>
-      </c>
-      <c r="R7" s="10" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="S7" s="10" t="inlineStr">
-        <is>
-          <t>只有两个交易日的低点，结构证据偏少。</t>
-        </is>
-      </c>
-      <c r="T7" s="10" t="inlineStr">
-        <is>
-          <t>后续只看是否跌破33.20。</t>
-        </is>
-      </c>
-      <c r="U7" s="11" t="inlineStr">
-        <is>
-          <t>箱体下沿需要多次确认、缩量反弹强弱</t>
-        </is>
-      </c>
-      <c r="V7" s="11" t="inlineStr">
-        <is>
-          <t>这是一条“暂时结构”，不是强结论。</t>
-        </is>
-      </c>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="10" t="n"/>
+      <c r="I7" s="10" t="n"/>
+      <c r="J7" s="10" t="n"/>
+      <c r="K7" s="10" t="n"/>
+      <c r="L7" s="10" t="n"/>
+      <c r="M7" s="10" t="n"/>
+      <c r="N7" s="10" t="n"/>
+      <c r="O7" s="10" t="n"/>
+      <c r="P7" s="10" t="n"/>
+      <c r="Q7" s="10" t="n"/>
+      <c r="R7" s="10" t="n"/>
+      <c r="S7" s="10" t="n"/>
+      <c r="T7" s="10" t="n"/>
+      <c r="U7" s="11" t="n"/>
+      <c r="V7" s="11" t="n"/>
       <c r="W7" s="26">
         <f>IF(B7="","",B7+3)</f>
         <v/>
@@ -1897,139 +1309,41 @@
         <f>IF(B7="","",(--(B7&lt;&gt;"")+--(C7&lt;&gt;"")+--(D7&lt;&gt;"")+--(E7&lt;&gt;"")+--(F7&lt;&gt;"")+--(G7&lt;&gt;"")+--(H7&lt;&gt;"")+--(I7&lt;&gt;"")+--(J7&lt;&gt;"")+--(K7&lt;&gt;"")+--(L7&lt;&gt;"")+--(M7&lt;&gt;"")+--(N7&lt;&gt;"")+--(O7&lt;&gt;"")+--(P7&lt;&gt;"")+--(Q7&lt;&gt;"")+--(R7&lt;&gt;"")+--(S7&lt;&gt;"")+--(T7&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA7" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AB7" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AC7" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AD7" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
+      <c r="AA7" s="18" t="n"/>
+      <c r="AB7" s="18" t="n"/>
+      <c r="AC7" s="18" t="n"/>
+      <c r="AD7" s="18" t="n"/>
       <c r="AE7" s="7">
         <f>IF(B7="","",IF(AND(AA7="合格",AB7="合格",AC7="合格",AD7="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="72" customHeight="1">
+    <row r="8">
       <c r="A8" s="7">
         <f>IF(B8="","",TEXT(B8,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B8" s="25" t="n">
-        <v>45842</v>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>半导体/封测</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>震荡偏强</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>震荡</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>同步板块</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>箱体下沿</t>
-        </is>
-      </c>
-      <c r="I8" s="10" t="inlineStr">
-        <is>
-          <t>33.20-33.30</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
-        <is>
-          <t>前两日33.23低点形成短线下沿，今日收33.23正好回到下沿。</t>
-        </is>
-      </c>
-      <c r="K8" s="10" t="inlineStr">
-        <is>
-          <t>接近</t>
-        </is>
-      </c>
-      <c r="L8" s="10" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="M8" s="10" t="inlineStr">
-        <is>
-          <t>横盘震荡</t>
-        </is>
-      </c>
-      <c r="N8" s="10" t="inlineStr">
-        <is>
-          <t>收33.23跌0.89%，最低33.10，成交量20.30万手；半导体跌0.93%，上证涨0.32%。</t>
-        </is>
-      </c>
-      <c r="O8" s="10" t="inlineStr">
-        <is>
-          <t>震荡整理</t>
-        </is>
-      </c>
-      <c r="P8" s="10" t="inlineStr">
-        <is>
-          <t>价格回到下沿附近但没有放量大跌，仍可能是箱体震荡；不过大盘上涨时个股不涨，主动性偏弱。</t>
-        </is>
-      </c>
-      <c r="Q8" s="10" t="inlineStr">
-        <is>
-          <t>如果下一日跌破33.00，震荡整理会转向突破失败或转弱。</t>
-        </is>
-      </c>
-      <c r="R8" s="10" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="S8" s="10" t="inlineStr">
-        <is>
-          <t>位置接近支撑但没有明确反包或放量，结论只能低强度。</t>
-        </is>
-      </c>
-      <c r="T8" s="10" t="inlineStr">
-        <is>
-          <t>后续只看是否跌破33.00。</t>
-        </is>
-      </c>
-      <c r="U8" s="11" t="inlineStr">
-        <is>
-          <t>弱于大盘的含义、箱体下沿有效性</t>
-        </is>
-      </c>
-      <c r="V8" s="11" t="inlineStr">
-        <is>
-          <t>这里更适合观察，不适合急着下强判断。</t>
-        </is>
-      </c>
+      <c r="B8" s="25" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
+      <c r="H8" s="10" t="n"/>
+      <c r="I8" s="10" t="n"/>
+      <c r="J8" s="10" t="n"/>
+      <c r="K8" s="10" t="n"/>
+      <c r="L8" s="10" t="n"/>
+      <c r="M8" s="10" t="n"/>
+      <c r="N8" s="10" t="n"/>
+      <c r="O8" s="10" t="n"/>
+      <c r="P8" s="10" t="n"/>
+      <c r="Q8" s="10" t="n"/>
+      <c r="R8" s="10" t="n"/>
+      <c r="S8" s="10" t="n"/>
+      <c r="T8" s="10" t="n"/>
+      <c r="U8" s="11" t="n"/>
+      <c r="V8" s="11" t="n"/>
       <c r="W8" s="26">
         <f>IF(B8="","",B8+3)</f>
         <v/>
@@ -2046,139 +1360,41 @@
         <f>IF(B8="","",(--(B8&lt;&gt;"")+--(C8&lt;&gt;"")+--(D8&lt;&gt;"")+--(E8&lt;&gt;"")+--(F8&lt;&gt;"")+--(G8&lt;&gt;"")+--(H8&lt;&gt;"")+--(I8&lt;&gt;"")+--(J8&lt;&gt;"")+--(K8&lt;&gt;"")+--(L8&lt;&gt;"")+--(M8&lt;&gt;"")+--(N8&lt;&gt;"")+--(O8&lt;&gt;"")+--(P8&lt;&gt;"")+--(Q8&lt;&gt;"")+--(R8&lt;&gt;"")+--(S8&lt;&gt;"")+--(T8&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA8" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AB8" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AC8" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AD8" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
+      <c r="AA8" s="18" t="n"/>
+      <c r="AB8" s="18" t="n"/>
+      <c r="AC8" s="18" t="n"/>
+      <c r="AD8" s="18" t="n"/>
       <c r="AE8" s="7">
         <f>IF(B8="","",IF(AND(AA8="合格",AB8="合格",AC8="合格",AD8="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="72" customHeight="1">
+    <row r="9">
       <c r="A9" s="7">
         <f>IF(B9="","",TEXT(B9,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B9" s="25" t="n">
-        <v>45845</v>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>半导体/封测</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>震荡偏强</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>震荡</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>弱于板块</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>大阳线低点</t>
-        </is>
-      </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>33.00</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
-        <is>
-          <t>6月27日放量阳线低点33.00，此前也作为回踩观察位。</t>
-        </is>
-      </c>
-      <c r="K9" s="10" t="inlineStr">
-        <is>
-          <t>跌破</t>
-        </is>
-      </c>
-      <c r="L9" s="10" t="inlineStr">
-        <is>
-          <t>清晰</t>
-        </is>
-      </c>
-      <c r="M9" s="10" t="inlineStr">
-        <is>
-          <t>跌破关键位</t>
-        </is>
-      </c>
-      <c r="N9" s="10" t="inlineStr">
-        <is>
-          <t>收32.95跌0.84%，最低32.88，跌破33.00，成交量15.46万手；半导体跌0.13%，上证微涨0.02%。</t>
-        </is>
-      </c>
-      <c r="O9" s="10" t="inlineStr">
-        <is>
-          <t>退潮转弱</t>
-        </is>
-      </c>
-      <c r="P9" s="10" t="inlineStr">
-        <is>
-          <t>在板块和大盘没有明显下跌时，个股跌破33.00关键位，说明前期突破结构被破坏。</t>
-        </is>
-      </c>
-      <c r="Q9" s="10" t="inlineStr">
-        <is>
-          <t>如果下一两日快速收回33.30上方，今天可能是假跌破。</t>
-        </is>
-      </c>
-      <c r="R9" s="10" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="S9" s="10" t="inlineStr">
-        <is>
-          <t>关键位清晰，且相对板块转弱，但缩量下跌意味着杀跌并不充分。</t>
-        </is>
-      </c>
-      <c r="T9" s="10" t="inlineStr">
-        <is>
-          <t>后续只看是否收回33.30。</t>
-        </is>
-      </c>
-      <c r="U9" s="11" t="inlineStr">
-        <is>
-          <t>跌破关键位、假跌破识别、相对弱势</t>
-        </is>
-      </c>
-      <c r="V9" s="11" t="inlineStr">
-        <is>
-          <t>这一天是从“支撑观察”转为“结构受损观察”的分界。</t>
-        </is>
-      </c>
+      <c r="B9" s="25" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
+      <c r="H9" s="10" t="n"/>
+      <c r="I9" s="10" t="n"/>
+      <c r="J9" s="10" t="n"/>
+      <c r="K9" s="10" t="n"/>
+      <c r="L9" s="10" t="n"/>
+      <c r="M9" s="10" t="n"/>
+      <c r="N9" s="10" t="n"/>
+      <c r="O9" s="10" t="n"/>
+      <c r="P9" s="10" t="n"/>
+      <c r="Q9" s="10" t="n"/>
+      <c r="R9" s="10" t="n"/>
+      <c r="S9" s="10" t="n"/>
+      <c r="T9" s="10" t="n"/>
+      <c r="U9" s="11" t="n"/>
+      <c r="V9" s="11" t="n"/>
       <c r="W9" s="26">
         <f>IF(B9="","",B9+3)</f>
         <v/>
@@ -2195,139 +1411,41 @@
         <f>IF(B9="","",(--(B9&lt;&gt;"")+--(C9&lt;&gt;"")+--(D9&lt;&gt;"")+--(E9&lt;&gt;"")+--(F9&lt;&gt;"")+--(G9&lt;&gt;"")+--(H9&lt;&gt;"")+--(I9&lt;&gt;"")+--(J9&lt;&gt;"")+--(K9&lt;&gt;"")+--(L9&lt;&gt;"")+--(M9&lt;&gt;"")+--(N9&lt;&gt;"")+--(O9&lt;&gt;"")+--(P9&lt;&gt;"")+--(Q9&lt;&gt;"")+--(R9&lt;&gt;"")+--(S9&lt;&gt;"")+--(T9&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA9" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AB9" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AC9" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AD9" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
+      <c r="AA9" s="18" t="n"/>
+      <c r="AB9" s="18" t="n"/>
+      <c r="AC9" s="18" t="n"/>
+      <c r="AD9" s="18" t="n"/>
       <c r="AE9" s="7">
         <f>IF(B9="","",IF(AND(AA9="合格",AB9="合格",AC9="合格",AD9="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="72" customHeight="1">
+    <row r="10">
       <c r="A10" s="7">
         <f>IF(B10="","",TEXT(B10,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B10" s="25" t="n">
-        <v>45846</v>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>半导体/封测</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>上升</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>轮动强势</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>同步板块</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>前高</t>
-        </is>
-      </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>33.30-33.40</t>
-        </is>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>跌破33.00后快速收回，33.30-33.40重新变成修复确认位。</t>
-        </is>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>跌破后收回</t>
-        </is>
-      </c>
-      <c r="L10" s="10" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="M10" s="10" t="inlineStr">
-        <is>
-          <t>低位反弹</t>
-        </is>
-      </c>
-      <c r="N10" s="10" t="inlineStr">
-        <is>
-          <t>收33.55涨1.82%，最低33.01后收回33.30-33.40，成交量24.45万手；半导体涨1.50%，上证涨0.70%。</t>
-        </is>
-      </c>
-      <c r="O10" s="10" t="inlineStr">
-        <is>
-          <t>弱反弹</t>
-        </is>
-      </c>
-      <c r="P10" s="10" t="inlineStr">
-        <is>
-          <t>价格收回关键位说明7月7日跌破没有继续恶化，但反弹主要伴随大盘和板块转强，暂不能认定重新启动。</t>
-        </is>
-      </c>
-      <c r="Q10" s="10" t="inlineStr">
-        <is>
-          <t>如果后续不能继续站稳33.40并上攻33.80，反弹仍可能只是箱体震荡的一部分。</t>
-        </is>
-      </c>
-      <c r="R10" s="10" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="S10" s="10" t="inlineStr">
-        <is>
-          <t>修复动作明确，但外部环境同步转强，个股独立性不足。</t>
-        </is>
-      </c>
-      <c r="T10" s="10" t="inlineStr">
-        <is>
-          <t>后续只看是否连续收在33.40上方。</t>
-        </is>
-      </c>
-      <c r="U10" s="11" t="inlineStr">
-        <is>
-          <t>跌破后收回、修复与重新启动区别</t>
-        </is>
-      </c>
-      <c r="V10" s="11" t="inlineStr">
-        <is>
-          <t>不要因为一天大涨就把它重新判成强趋势。</t>
-        </is>
-      </c>
+      <c r="B10" s="25" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="10" t="n"/>
+      <c r="I10" s="10" t="n"/>
+      <c r="J10" s="10" t="n"/>
+      <c r="K10" s="10" t="n"/>
+      <c r="L10" s="10" t="n"/>
+      <c r="M10" s="10" t="n"/>
+      <c r="N10" s="10" t="n"/>
+      <c r="O10" s="10" t="n"/>
+      <c r="P10" s="10" t="n"/>
+      <c r="Q10" s="10" t="n"/>
+      <c r="R10" s="10" t="n"/>
+      <c r="S10" s="10" t="n"/>
+      <c r="T10" s="10" t="n"/>
+      <c r="U10" s="11" t="n"/>
+      <c r="V10" s="11" t="n"/>
       <c r="W10" s="26">
         <f>IF(B10="","",B10+3)</f>
         <v/>
@@ -2344,139 +1462,41 @@
         <f>IF(B10="","",(--(B10&lt;&gt;"")+--(C10&lt;&gt;"")+--(D10&lt;&gt;"")+--(E10&lt;&gt;"")+--(F10&lt;&gt;"")+--(G10&lt;&gt;"")+--(H10&lt;&gt;"")+--(I10&lt;&gt;"")+--(J10&lt;&gt;"")+--(K10&lt;&gt;"")+--(L10&lt;&gt;"")+--(M10&lt;&gt;"")+--(N10&lt;&gt;"")+--(O10&lt;&gt;"")+--(P10&lt;&gt;"")+--(Q10&lt;&gt;"")+--(R10&lt;&gt;"")+--(S10&lt;&gt;"")+--(T10&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA10" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AB10" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AC10" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AD10" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
+      <c r="AA10" s="18" t="n"/>
+      <c r="AB10" s="18" t="n"/>
+      <c r="AC10" s="18" t="n"/>
+      <c r="AD10" s="18" t="n"/>
       <c r="AE10" s="7">
         <f>IF(B10="","",IF(AND(AA10="合格",AB10="合格",AC10="合格",AD10="合格"),"有效","无效"))</f>
         <v/>
       </c>
     </row>
-    <row r="11" ht="72" customHeight="1">
+    <row r="11">
       <c r="A11" s="7">
         <f>IF(B11="","",TEXT(B11,"yyyymmdd")&amp;"-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B11" s="25" t="n">
-        <v>45847</v>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>半导体/封测</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>震荡偏强</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>震荡</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>同步板块</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>箱体下沿</t>
-        </is>
-      </c>
-      <c r="I11" s="10" t="inlineStr">
-        <is>
-          <t>33.00-33.20</t>
-        </is>
-      </c>
-      <c r="J11" s="10" t="inlineStr">
-        <is>
-          <t>近几日低点集中在33.00-33.20，当前仍围绕这个区域反复。</t>
-        </is>
-      </c>
-      <c r="K11" s="10" t="inlineStr">
-        <is>
-          <t>接近</t>
-        </is>
-      </c>
-      <c r="L11" s="10" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="M11" s="10" t="inlineStr">
-        <is>
-          <t>横盘震荡</t>
-        </is>
-      </c>
-      <c r="N11" s="10" t="inlineStr">
-        <is>
-          <t>收33.18跌1.10%，最低33.10，成交量19.43万手；半导体跌1.12%，上证跌0.13%。</t>
-        </is>
-      </c>
-      <c r="O11" s="10" t="inlineStr">
-        <is>
-          <t>震荡整理</t>
-        </is>
-      </c>
-      <c r="P11" s="10" t="inlineStr">
-        <is>
-          <t>价格没有继续向上确认33.40，也没有有效跌破33.00，说明短线仍在33.00-34.08之间震荡。</t>
-        </is>
-      </c>
-      <c r="Q11" s="10" t="inlineStr">
-        <is>
-          <t>如果后续放量跌破33.00，震荡整理会转为转弱；若放量站上34.08，才说明重新转强。</t>
-        </is>
-      </c>
-      <c r="R11" s="10" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="S11" s="10" t="inlineStr">
-        <is>
-          <t>上下边界都有，但当前价格在中低位，方向信息不足。</t>
-        </is>
-      </c>
-      <c r="T11" s="10" t="inlineStr">
-        <is>
-          <t>后续只看33.00是否被有效跌破。</t>
-        </is>
-      </c>
-      <c r="U11" s="11" t="inlineStr">
-        <is>
-          <t>箱体边界、方向未明时降低判断强度</t>
-        </is>
-      </c>
-      <c r="V11" s="11" t="inlineStr">
-        <is>
-          <t>这是一个“看不清就承认看不清”的样本。</t>
-        </is>
-      </c>
+      <c r="B11" s="25" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
+      <c r="H11" s="10" t="n"/>
+      <c r="I11" s="10" t="n"/>
+      <c r="J11" s="10" t="n"/>
+      <c r="K11" s="10" t="n"/>
+      <c r="L11" s="10" t="n"/>
+      <c r="M11" s="10" t="n"/>
+      <c r="N11" s="10" t="n"/>
+      <c r="O11" s="10" t="n"/>
+      <c r="P11" s="10" t="n"/>
+      <c r="Q11" s="10" t="n"/>
+      <c r="R11" s="10" t="n"/>
+      <c r="S11" s="10" t="n"/>
+      <c r="T11" s="10" t="n"/>
+      <c r="U11" s="11" t="n"/>
+      <c r="V11" s="11" t="n"/>
       <c r="W11" s="26">
         <f>IF(B11="","",B11+3)</f>
         <v/>
@@ -2493,26 +1513,10 @@
         <f>IF(B11="","",(--(B11&lt;&gt;"")+--(C11&lt;&gt;"")+--(D11&lt;&gt;"")+--(E11&lt;&gt;"")+--(F11&lt;&gt;"")+--(G11&lt;&gt;"")+--(H11&lt;&gt;"")+--(I11&lt;&gt;"")+--(J11&lt;&gt;"")+--(K11&lt;&gt;"")+--(L11&lt;&gt;"")+--(M11&lt;&gt;"")+--(N11&lt;&gt;"")+--(O11&lt;&gt;"")+--(P11&lt;&gt;"")+--(Q11&lt;&gt;"")+--(R11&lt;&gt;"")+--(S11&lt;&gt;"")+--(T11&lt;&gt;""))/19)</f>
         <v/>
       </c>
-      <c r="AA11" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AB11" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AC11" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
-      <c r="AD11" s="18" t="inlineStr">
-        <is>
-          <t>合格</t>
-        </is>
-      </c>
+      <c r="AA11" s="18" t="n"/>
+      <c r="AB11" s="18" t="n"/>
+      <c r="AC11" s="18" t="n"/>
+      <c r="AD11" s="18" t="n"/>
       <c r="AE11" s="7">
         <f>IF(B11="","",IF(AND(AA11="合格",AB11="合格",AC11="合格",AD11="合格"),"有效","无效"))</f>
         <v/>
@@ -28464,817 +27468,229 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="72" customHeight="1">
+    <row r="2">
       <c r="A2" s="15">
         <f>IF(B2="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>20250626-001</t>
-        </is>
-      </c>
-      <c r="C2" s="28" t="n">
-        <v>45834</v>
-      </c>
-      <c r="D2" s="18" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="E2" s="18" t="inlineStr">
-        <is>
-          <t>前高</t>
-        </is>
-      </c>
-      <c r="F2" s="18" t="inlineStr">
-        <is>
-          <t>33.30-33.40</t>
-        </is>
-      </c>
-      <c r="G2" s="18" t="inlineStr">
-        <is>
-          <t>冲高回落</t>
-        </is>
-      </c>
-      <c r="H2" s="18" t="inlineStr">
-        <is>
-          <t>高位分歧</t>
-        </is>
-      </c>
-      <c r="I2" s="18" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="J2" s="18" t="inlineStr">
-        <is>
-          <t>后续只看是否收盘重新站上33.40。</t>
-        </is>
-      </c>
-      <c r="K2" s="18" t="inlineStr">
-        <is>
-          <t>3日</t>
-        </is>
-      </c>
-      <c r="L2" s="28" t="n">
-        <v>45839</v>
-      </c>
-      <c r="M2" s="18" t="inlineStr">
-        <is>
-          <t>收33.97，盘中34.38，已重新站上33.40但没有收过34.08。</t>
-        </is>
-      </c>
-      <c r="N2" s="18" t="inlineStr">
-        <is>
-          <t>向上延续</t>
-        </is>
-      </c>
-      <c r="O2" s="18" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="P2" s="18" t="inlineStr">
-        <is>
-          <t>出现</t>
-        </is>
-      </c>
-      <c r="Q2" s="18" t="inlineStr">
-        <is>
-          <t>削弱</t>
-        </is>
-      </c>
-      <c r="R2" s="18" t="inlineStr">
-        <is>
-          <t>过程合理</t>
-        </is>
-      </c>
-      <c r="S2" s="18" t="inlineStr">
-        <is>
-          <t>概率结果失败</t>
-        </is>
-      </c>
-      <c r="T2" s="18" t="inlineStr">
-        <is>
-          <t>前高分歧不等于失败，必须等收盘确认。</t>
-        </is>
-      </c>
-      <c r="U2" s="18" t="inlineStr">
-        <is>
-          <t>收盘确认与盘中突破区别</t>
-        </is>
-      </c>
+      <c r="B2" s="18" t="n"/>
+      <c r="C2" s="28" t="n"/>
+      <c r="D2" s="18" t="n"/>
+      <c r="E2" s="18" t="n"/>
+      <c r="F2" s="18" t="n"/>
+      <c r="G2" s="18" t="n"/>
+      <c r="H2" s="18" t="n"/>
+      <c r="I2" s="18" t="n"/>
+      <c r="J2" s="18" t="n"/>
+      <c r="K2" s="18" t="n"/>
+      <c r="L2" s="28" t="n"/>
+      <c r="M2" s="18" t="n"/>
+      <c r="N2" s="18" t="n"/>
+      <c r="O2" s="18" t="n"/>
+      <c r="P2" s="18" t="n"/>
+      <c r="Q2" s="18" t="n"/>
+      <c r="R2" s="18" t="n"/>
+      <c r="S2" s="18" t="n"/>
+      <c r="T2" s="18" t="n"/>
+      <c r="U2" s="18" t="n"/>
       <c r="V2" s="29">
         <f>IF(L2="","",IF(TODAY()&gt;=L2,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W2" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="X2" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="72" customHeight="1">
+      <c r="W2" s="18" t="n"/>
+      <c r="X2" s="18" t="n"/>
+    </row>
+    <row r="3">
       <c r="A3" s="15">
         <f>IF(B3="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B3" s="18" t="inlineStr">
-        <is>
-          <t>20250627-002</t>
-        </is>
-      </c>
-      <c r="C3" s="28" t="n">
-        <v>45835</v>
-      </c>
-      <c r="D3" s="18" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="E3" s="18" t="inlineStr">
-        <is>
-          <t>前高</t>
-        </is>
-      </c>
-      <c r="F3" s="18" t="inlineStr">
-        <is>
-          <t>33.40</t>
-        </is>
-      </c>
-      <c r="G3" s="18" t="inlineStr">
-        <is>
-          <t>放量突破</t>
-        </is>
-      </c>
-      <c r="H3" s="18" t="inlineStr">
-        <is>
-          <t>真突破/启动尝试</t>
-        </is>
-      </c>
-      <c r="I3" s="18" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="J3" s="18" t="inlineStr">
-        <is>
-          <t>后续只看是否守住33.30-33.40。</t>
-        </is>
-      </c>
-      <c r="K3" s="18" t="inlineStr">
-        <is>
-          <t>3日</t>
-        </is>
-      </c>
-      <c r="L3" s="28" t="n">
-        <v>45840</v>
-      </c>
-      <c r="M3" s="18" t="inlineStr">
-        <is>
-          <t>收33.31，基本回踩到33.30附近，未明显跌破但突破延续不足。</t>
-        </is>
-      </c>
-      <c r="N3" s="18" t="inlineStr">
-        <is>
-          <t>震荡消化</t>
-        </is>
-      </c>
-      <c r="O3" s="18" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="P3" s="18" t="inlineStr">
-        <is>
-          <t>部分出现</t>
-        </is>
-      </c>
-      <c r="Q3" s="18" t="inlineStr">
-        <is>
-          <t>削弱</t>
-        </is>
-      </c>
-      <c r="R3" s="18" t="inlineStr">
-        <is>
-          <t>过程合理</t>
-        </is>
-      </c>
-      <c r="S3" s="18" t="inlineStr">
-        <is>
-          <t>无明显错误</t>
-        </is>
-      </c>
-      <c r="T3" s="18" t="inlineStr">
-        <is>
-          <t>突破后如果不能继续放量，先按震荡消化处理。</t>
-        </is>
-      </c>
-      <c r="U3" s="18" t="inlineStr">
-        <is>
-          <t>突破后的回踩确认</t>
-        </is>
-      </c>
+      <c r="B3" s="18" t="n"/>
+      <c r="C3" s="28" t="n"/>
+      <c r="D3" s="18" t="n"/>
+      <c r="E3" s="18" t="n"/>
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="18" t="n"/>
+      <c r="H3" s="18" t="n"/>
+      <c r="I3" s="18" t="n"/>
+      <c r="J3" s="18" t="n"/>
+      <c r="K3" s="18" t="n"/>
+      <c r="L3" s="28" t="n"/>
+      <c r="M3" s="18" t="n"/>
+      <c r="N3" s="18" t="n"/>
+      <c r="O3" s="18" t="n"/>
+      <c r="P3" s="18" t="n"/>
+      <c r="Q3" s="18" t="n"/>
+      <c r="R3" s="18" t="n"/>
+      <c r="S3" s="18" t="n"/>
+      <c r="T3" s="18" t="n"/>
+      <c r="U3" s="18" t="n"/>
       <c r="V3" s="29">
         <f>IF(L3="","",IF(TODAY()&gt;=L3,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W3" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="X3" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="72" customHeight="1">
+      <c r="W3" s="18" t="n"/>
+      <c r="X3" s="18" t="n"/>
+    </row>
+    <row r="4">
       <c r="A4" s="15">
         <f>IF(B4="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B4" s="18" t="inlineStr">
-        <is>
-          <t>20250630-003</t>
-        </is>
-      </c>
-      <c r="C4" s="28" t="n">
-        <v>45838</v>
-      </c>
-      <c r="D4" s="18" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="E4" s="18" t="inlineStr">
-        <is>
-          <t>前高</t>
-        </is>
-      </c>
-      <c r="F4" s="18" t="inlineStr">
-        <is>
-          <t>34.08</t>
-        </is>
-      </c>
-      <c r="G4" s="18" t="inlineStr">
-        <is>
-          <t>横盘震荡</t>
-        </is>
-      </c>
-      <c r="H4" s="18" t="inlineStr">
-        <is>
-          <t>震荡整理</t>
-        </is>
-      </c>
-      <c r="I4" s="18" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="J4" s="18" t="inlineStr">
-        <is>
-          <t>后续只看是否收盘站上34.08。</t>
-        </is>
-      </c>
-      <c r="K4" s="18" t="inlineStr">
-        <is>
-          <t>3日</t>
-        </is>
-      </c>
-      <c r="L4" s="28" t="n">
-        <v>45841</v>
-      </c>
-      <c r="M4" s="18" t="inlineStr">
-        <is>
-          <t>收33.53，未站上34.08，仍在33.20-34.08之间。</t>
-        </is>
-      </c>
-      <c r="N4" s="18" t="inlineStr">
-        <is>
-          <t>震荡消化</t>
-        </is>
-      </c>
-      <c r="O4" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="P4" s="18" t="inlineStr">
-        <is>
-          <t>未出现</t>
-        </is>
-      </c>
-      <c r="Q4" s="18" t="inlineStr">
-        <is>
-          <t>强化</t>
-        </is>
-      </c>
-      <c r="R4" s="18" t="inlineStr">
-        <is>
-          <t>过程合理</t>
-        </is>
-      </c>
-      <c r="S4" s="18" t="inlineStr">
-        <is>
-          <t>无明显错误</t>
-        </is>
-      </c>
-      <c r="T4" s="18" t="inlineStr">
-        <is>
-          <t>低强度震荡判断可以接受，不需要硬预测方向。</t>
-        </is>
-      </c>
-      <c r="U4" s="18" t="inlineStr">
-        <is>
-          <t>箱体上沿确认</t>
-        </is>
-      </c>
+      <c r="B4" s="18" t="n"/>
+      <c r="C4" s="28" t="n"/>
+      <c r="D4" s="18" t="n"/>
+      <c r="E4" s="18" t="n"/>
+      <c r="F4" s="18" t="n"/>
+      <c r="G4" s="18" t="n"/>
+      <c r="H4" s="18" t="n"/>
+      <c r="I4" s="18" t="n"/>
+      <c r="J4" s="18" t="n"/>
+      <c r="K4" s="18" t="n"/>
+      <c r="L4" s="28" t="n"/>
+      <c r="M4" s="18" t="n"/>
+      <c r="N4" s="18" t="n"/>
+      <c r="O4" s="18" t="n"/>
+      <c r="P4" s="18" t="n"/>
+      <c r="Q4" s="18" t="n"/>
+      <c r="R4" s="18" t="n"/>
+      <c r="S4" s="18" t="n"/>
+      <c r="T4" s="18" t="n"/>
+      <c r="U4" s="18" t="n"/>
       <c r="V4" s="29">
         <f>IF(L4="","",IF(TODAY()&gt;=L4,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W4" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="X4" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="72" customHeight="1">
+      <c r="W4" s="18" t="n"/>
+      <c r="X4" s="18" t="n"/>
+    </row>
+    <row r="5">
       <c r="A5" s="15">
         <f>IF(B5="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>20250701-004</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="n">
-        <v>45839</v>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>前高</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>34.08</t>
-        </is>
-      </c>
-      <c r="G5" s="18" t="inlineStr">
-        <is>
-          <t>高位放量震荡</t>
-        </is>
-      </c>
-      <c r="H5" s="18" t="inlineStr">
-        <is>
-          <t>高位分歧</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="J5" s="18" t="inlineStr">
-        <is>
-          <t>后续只看是否收盘站上34.08。</t>
-        </is>
-      </c>
-      <c r="K5" s="18" t="inlineStr">
-        <is>
-          <t>3日</t>
-        </is>
-      </c>
-      <c r="L5" s="28" t="n">
-        <v>45842</v>
-      </c>
-      <c r="M5" s="18" t="inlineStr">
-        <is>
-          <t>收33.23，没有站回34.08，反而回到短线下沿。</t>
-        </is>
-      </c>
-      <c r="N5" s="18" t="inlineStr">
-        <is>
-          <t>冲高回落</t>
-        </is>
-      </c>
-      <c r="O5" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="P5" s="18" t="inlineStr">
-        <is>
-          <t>未出现</t>
-        </is>
-      </c>
-      <c r="Q5" s="18" t="inlineStr">
-        <is>
-          <t>强化</t>
-        </is>
-      </c>
-      <c r="R5" s="18" t="inlineStr">
-        <is>
-          <t>过程合理</t>
-        </is>
-      </c>
-      <c r="S5" s="18" t="inlineStr">
-        <is>
-          <t>无明显错误</t>
-        </is>
-      </c>
-      <c r="T5" s="18" t="inlineStr">
-        <is>
-          <t>盘中新高不如收盘站稳重要。</t>
-        </is>
-      </c>
-      <c r="U5" s="18" t="inlineStr">
-        <is>
-          <t>假突破与分歧换手区分</t>
-        </is>
-      </c>
+      <c r="B5" s="18" t="n"/>
+      <c r="C5" s="28" t="n"/>
+      <c r="D5" s="18" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
+      <c r="K5" s="18" t="n"/>
+      <c r="L5" s="28" t="n"/>
+      <c r="M5" s="18" t="n"/>
+      <c r="N5" s="18" t="n"/>
+      <c r="O5" s="18" t="n"/>
+      <c r="P5" s="18" t="n"/>
+      <c r="Q5" s="18" t="n"/>
+      <c r="R5" s="18" t="n"/>
+      <c r="S5" s="18" t="n"/>
+      <c r="T5" s="18" t="n"/>
+      <c r="U5" s="18" t="n"/>
       <c r="V5" s="29">
         <f>IF(L5="","",IF(TODAY()&gt;=L5,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W5" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="X5" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="72" customHeight="1">
+      <c r="W5" s="18" t="n"/>
+      <c r="X5" s="18" t="n"/>
+    </row>
+    <row r="6">
       <c r="A6" s="15">
         <f>IF(B6="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>20250702-005</t>
-        </is>
-      </c>
-      <c r="C6" s="28" t="n">
-        <v>45840</v>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>大阳线低点</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>33.00-33.30</t>
-        </is>
-      </c>
-      <c r="G6" s="18" t="inlineStr">
-        <is>
-          <t>缩量回调</t>
-        </is>
-      </c>
-      <c r="H6" s="18" t="inlineStr">
-        <is>
-          <t>健康回调</t>
-        </is>
-      </c>
-      <c r="I6" s="18" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="J6" s="18" t="inlineStr">
-        <is>
-          <t>后续只看是否跌破33.00。</t>
-        </is>
-      </c>
-      <c r="K6" s="18" t="inlineStr">
-        <is>
-          <t>3日</t>
-        </is>
-      </c>
-      <c r="L6" s="28" t="n">
-        <v>45845</v>
-      </c>
-      <c r="M6" s="18" t="inlineStr">
-        <is>
-          <t>收32.95，跌破33.00，但成交量继续缩小。</t>
-        </is>
-      </c>
-      <c r="N6" s="18" t="inlineStr">
-        <is>
-          <t>跌破支撑</t>
-        </is>
-      </c>
-      <c r="O6" s="18" t="inlineStr">
-        <is>
-          <t>一般</t>
-        </is>
-      </c>
-      <c r="P6" s="18" t="inlineStr">
-        <is>
-          <t>出现</t>
-        </is>
-      </c>
-      <c r="Q6" s="18" t="inlineStr">
-        <is>
-          <t>证伪</t>
-        </is>
-      </c>
-      <c r="R6" s="18" t="inlineStr">
-        <is>
-          <t>概率失败</t>
-        </is>
-      </c>
-      <c r="S6" s="18" t="inlineStr">
-        <is>
-          <t>概率结果失败</t>
-        </is>
-      </c>
-      <c r="T6" s="18" t="inlineStr">
-        <is>
-          <t>健康回调假设被证伪时要切换解释，不要补理由。</t>
-        </is>
-      </c>
-      <c r="U6" s="18" t="inlineStr">
-        <is>
-          <t>支撑区间有效性</t>
-        </is>
-      </c>
+      <c r="B6" s="18" t="n"/>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="18" t="n"/>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="18" t="n"/>
+      <c r="J6" s="18" t="n"/>
+      <c r="K6" s="18" t="n"/>
+      <c r="L6" s="28" t="n"/>
+      <c r="M6" s="18" t="n"/>
+      <c r="N6" s="18" t="n"/>
+      <c r="O6" s="18" t="n"/>
+      <c r="P6" s="18" t="n"/>
+      <c r="Q6" s="18" t="n"/>
+      <c r="R6" s="18" t="n"/>
+      <c r="S6" s="18" t="n"/>
+      <c r="T6" s="18" t="n"/>
+      <c r="U6" s="18" t="n"/>
       <c r="V6" s="29">
         <f>IF(L6="","",IF(TODAY()&gt;=L6,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W6" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="X6" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="72" customHeight="1">
+      <c r="W6" s="18" t="n"/>
+      <c r="X6" s="18" t="n"/>
+    </row>
+    <row r="7">
       <c r="A7" s="15">
         <f>IF(B7="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>20250703-006</t>
-        </is>
-      </c>
-      <c r="C7" s="28" t="n">
-        <v>45841</v>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>箱体下沿</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>33.20-33.30</t>
-        </is>
-      </c>
-      <c r="G7" s="18" t="inlineStr">
-        <is>
-          <t>回踩支撑不破</t>
-        </is>
-      </c>
-      <c r="H7" s="18" t="inlineStr">
-        <is>
-          <t>震荡整理</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="J7" s="18" t="inlineStr">
-        <is>
-          <t>后续只看是否跌破33.20。</t>
-        </is>
-      </c>
-      <c r="K7" s="18" t="inlineStr">
-        <is>
-          <t>3日</t>
-        </is>
-      </c>
-      <c r="L7" s="28" t="n">
-        <v>45846</v>
-      </c>
-      <c r="M7" s="18" t="inlineStr">
-        <is>
-          <t>收33.55，未跌破33.20，并重新收回33.40上方。</t>
-        </is>
-      </c>
-      <c r="N7" s="18" t="inlineStr">
-        <is>
-          <t>修复转强</t>
-        </is>
-      </c>
-      <c r="O7" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="P7" s="18" t="inlineStr">
-        <is>
-          <t>未出现</t>
-        </is>
-      </c>
-      <c r="Q7" s="18" t="inlineStr">
-        <is>
-          <t>强化</t>
-        </is>
-      </c>
-      <c r="R7" s="18" t="inlineStr">
-        <is>
-          <t>过程合理</t>
-        </is>
-      </c>
-      <c r="S7" s="18" t="inlineStr">
-        <is>
-          <t>无明显错误</t>
-        </is>
-      </c>
-      <c r="T7" s="18" t="inlineStr">
-        <is>
-          <t>两个低点形成的临时箱体可以观察，但强度要低。</t>
-        </is>
-      </c>
-      <c r="U7" s="18" t="inlineStr">
-        <is>
-          <t>临时箱体识别</t>
-        </is>
-      </c>
+      <c r="B7" s="18" t="n"/>
+      <c r="C7" s="28" t="n"/>
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="28" t="n"/>
+      <c r="M7" s="18" t="n"/>
+      <c r="N7" s="18" t="n"/>
+      <c r="O7" s="18" t="n"/>
+      <c r="P7" s="18" t="n"/>
+      <c r="Q7" s="18" t="n"/>
+      <c r="R7" s="18" t="n"/>
+      <c r="S7" s="18" t="n"/>
+      <c r="T7" s="18" t="n"/>
+      <c r="U7" s="18" t="n"/>
       <c r="V7" s="29">
         <f>IF(L7="","",IF(TODAY()&gt;=L7,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W7" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="X7" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="72" customHeight="1">
+      <c r="W7" s="18" t="n"/>
+      <c r="X7" s="18" t="n"/>
+    </row>
+    <row r="8">
       <c r="A8" s="15">
         <f>IF(B8="","","V-"&amp;TEXT(ROW()-1,"000"))</f>
         <v/>
       </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>20250704-007</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="n">
-        <v>45842</v>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>长电科技 600584.SH</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>箱体下沿</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>33.20-33.30</t>
-        </is>
-      </c>
-      <c r="G8" s="18" t="inlineStr">
-        <is>
-          <t>横盘震荡</t>
-        </is>
-      </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>震荡整理</t>
-        </is>
-      </c>
-      <c r="I8" s="18" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="J8" s="18" t="inlineStr">
-        <is>
-          <t>后续只看是否跌破33.00。</t>
-        </is>
-      </c>
-      <c r="K8" s="18" t="inlineStr">
-        <is>
-          <t>3日</t>
-        </is>
-      </c>
-      <c r="L8" s="28" t="n">
-        <v>45847</v>
-      </c>
-      <c r="M8" s="18" t="inlineStr">
-        <is>
-          <t>收33.18，未跌破33.00，但也没有向上确认。</t>
-        </is>
-      </c>
-      <c r="N8" s="18" t="inlineStr">
-        <is>
-          <t>震荡消化</t>
-        </is>
-      </c>
-      <c r="O8" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="P8" s="18" t="inlineStr">
-        <is>
-          <t>未出现</t>
-        </is>
-      </c>
-      <c r="Q8" s="18" t="inlineStr">
-        <is>
-          <t>仍不确定</t>
-        </is>
-      </c>
-      <c r="R8" s="18" t="inlineStr">
-        <is>
-          <t>过程合理</t>
-        </is>
-      </c>
-      <c r="S8" s="18" t="inlineStr">
-        <is>
-          <t>无明显错误</t>
-        </is>
-      </c>
-      <c r="T8" s="18" t="inlineStr">
-        <is>
-          <t>低强度判断允许保持不确定，不必强行改成看多或看空。</t>
-        </is>
-      </c>
-      <c r="U8" s="18" t="inlineStr">
-        <is>
-          <t>方向不明时的观察纪律</t>
-        </is>
-      </c>
+      <c r="B8" s="18" t="n"/>
+      <c r="C8" s="28" t="n"/>
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="18" t="n"/>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="18" t="n"/>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="18" t="n"/>
+      <c r="L8" s="28" t="n"/>
+      <c r="M8" s="18" t="n"/>
+      <c r="N8" s="18" t="n"/>
+      <c r="O8" s="18" t="n"/>
+      <c r="P8" s="18" t="n"/>
+      <c r="Q8" s="18" t="n"/>
+      <c r="R8" s="18" t="n"/>
+      <c r="S8" s="18" t="n"/>
+      <c r="T8" s="18" t="n"/>
+      <c r="U8" s="18" t="n"/>
       <c r="V8" s="29">
         <f>IF(L8="","",IF(TODAY()&gt;=L8,"到期","未到期"))</f>
         <v/>
       </c>
-      <c r="W8" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="X8" s="18" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
+      <c r="W8" s="18" t="n"/>
+      <c r="X8" s="18" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15">

</xml_diff>